<commit_message>
Conform the research model's display precision and widths to the spec; add figure c's on-chart note
Gap per patient and the test 2 slope display to 1 decimal, dollars per day to
cents, test 1 shares and drops to 0.1 point (spec Precision); wider label
columns so no text clips. Figure source lines use the spec's wording
(Healthcare Utilization Reports); figure c carries the spec's note on the
chart. No value or verdict changed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/capabilities/economic-research/model.xlsx
+++ b/capabilities/economic-research/model.xlsx
@@ -167,7 +167,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -192,18 +192,17 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -574,7 +573,7 @@
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -1894,7 +1893,7 @@
   <dimension ref="A1:U17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
@@ -2044,7 +2043,7 @@
         <f>INDEX(WL_PATIENTS,1)*BENCH_DAYS</f>
         <v>86618.0</v>
       </c>
-      <c r="D4" s="18">
+      <c r="D4" s="16">
         <f>INDEX(DAYS_PER_PT,1)-BENCH_DAYS</f>
         <v>-4.064651689025375</v>
       </c>
@@ -2060,7 +2059,7 @@
         <f>INDEX(WL_DAYS,1)-INDEX(EXCESS_DAYS,1)</f>
         <v>61470.0</v>
       </c>
-      <c r="H4" s="19">
+      <c r="H4" s="18">
         <f>INDEX(EXCESS_DAYS,1)/INDEX(WL_DAYS,1)</f>
         <v>0.0</v>
       </c>
@@ -2080,31 +2079,31 @@
         <f>INDEX(REASON_NO_BED,1)+INDEX(REASON_BEHAVIOR,1)+INDEX(REASON_SPECIAL_CARE,1)+INDEX(REASON_FINANCIAL,1)+INDEX(REASON_GUARDIANSHIP,1)+INDEX(REASON_PASARR,1)+INDEX(REASON_OTHER,1)</f>
         <v>120.0</v>
       </c>
-      <c r="M4" s="19">
+      <c r="M4" s="18">
         <f>INDEX(REASON_NO_BED,1)/INDEX(REASON_SUM,1)</f>
         <v>0.325</v>
       </c>
-      <c r="N4" s="19">
+      <c r="N4" s="18">
         <f>INDEX(REASON_BEHAVIOR,1)/INDEX(REASON_SUM,1)</f>
         <v>0.13333333333333333</v>
       </c>
-      <c r="O4" s="19">
+      <c r="O4" s="18">
         <f>INDEX(REASON_SPECIAL_CARE,1)/INDEX(REASON_SUM,1)</f>
         <v>0.19166666666666668</v>
       </c>
-      <c r="P4" s="19">
+      <c r="P4" s="18">
         <f>INDEX(REASON_FINANCIAL,1)/INDEX(REASON_SUM,1)</f>
         <v>0.15</v>
       </c>
-      <c r="Q4" s="19">
+      <c r="Q4" s="18">
         <f>INDEX(REASON_GUARDIANSHIP,1)/INDEX(REASON_SUM,1)</f>
         <v>0.09166666666666666</v>
       </c>
-      <c r="R4" s="19">
+      <c r="R4" s="18">
         <f>INDEX(REASON_PASARR,1)/INDEX(REASON_SUM,1)</f>
         <v>0.016666666666666666</v>
       </c>
-      <c r="S4" s="19">
+      <c r="S4" s="18">
         <f>INDEX(REASON_OTHER,1)/INDEX(REASON_SUM,1)</f>
         <v>0.09166666666666666</v>
       </c>
@@ -2130,7 +2129,7 @@
         <f>INDEX(WL_PATIENTS,2)*BENCH_DAYS</f>
         <v>74116.0</v>
       </c>
-      <c r="D5" s="18">
+      <c r="D5" s="16">
         <f>INDEX(DAYS_PER_PT,2)-BENCH_DAYS</f>
         <v>-1.5158670192670947</v>
       </c>
@@ -2146,7 +2145,7 @@
         <f>INDEX(WL_DAYS,2)-INDEX(EXCESS_DAYS,2)</f>
         <v>66091.0</v>
       </c>
-      <c r="H5" s="19">
+      <c r="H5" s="18">
         <f>INDEX(EXCESS_DAYS,2)/INDEX(WL_DAYS,2)</f>
         <v>0.0</v>
       </c>
@@ -2166,31 +2165,31 @@
         <f>INDEX(REASON_NO_BED,2)+INDEX(REASON_BEHAVIOR,2)+INDEX(REASON_SPECIAL_CARE,2)+INDEX(REASON_FINANCIAL,2)+INDEX(REASON_GUARDIANSHIP,2)+INDEX(REASON_PASARR,2)+INDEX(REASON_OTHER,2)</f>
         <v>171.0</v>
       </c>
-      <c r="M5" s="19">
+      <c r="M5" s="18">
         <f>INDEX(REASON_NO_BED,2)/INDEX(REASON_SUM,2)</f>
         <v>0.3333333333333333</v>
       </c>
-      <c r="N5" s="19">
+      <c r="N5" s="18">
         <f>INDEX(REASON_BEHAVIOR,2)/INDEX(REASON_SUM,2)</f>
         <v>0.1695906432748538</v>
       </c>
-      <c r="O5" s="19">
+      <c r="O5" s="18">
         <f>INDEX(REASON_SPECIAL_CARE,2)/INDEX(REASON_SUM,2)</f>
         <v>0.09941520467836257</v>
       </c>
-      <c r="P5" s="19">
+      <c r="P5" s="18">
         <f>INDEX(REASON_FINANCIAL,2)/INDEX(REASON_SUM,2)</f>
         <v>0.18128654970760233</v>
       </c>
-      <c r="Q5" s="19">
+      <c r="Q5" s="18">
         <f>INDEX(REASON_GUARDIANSHIP,2)/INDEX(REASON_SUM,2)</f>
         <v>0.10526315789473684</v>
       </c>
-      <c r="R5" s="19">
+      <c r="R5" s="18">
         <f>INDEX(REASON_PASARR,2)/INDEX(REASON_SUM,2)</f>
         <v>0.011695906432748537</v>
       </c>
-      <c r="S5" s="19">
+      <c r="S5" s="18">
         <f>INDEX(REASON_OTHER,2)/INDEX(REASON_SUM,2)</f>
         <v>0.09941520467836257</v>
       </c>
@@ -2216,7 +2215,7 @@
         <f>INDEX(WL_PATIENTS,3)*BENCH_DAYS</f>
         <v>67060.0</v>
       </c>
-      <c r="D6" s="18">
+      <c r="D6" s="16">
         <f>INDEX(DAYS_PER_PT,3)-BENCH_DAYS</f>
         <v>2.474112734864299</v>
       </c>
@@ -2232,7 +2231,7 @@
         <f>INDEX(WL_DAYS,3)-INDEX(EXCESS_DAYS,3)</f>
         <v>67060.0</v>
       </c>
-      <c r="H6" s="19">
+      <c r="H6" s="18">
         <f>INDEX(EXCESS_DAYS,3)/INDEX(WL_DAYS,3)</f>
         <v>0.1501818504391023</v>
       </c>
@@ -2252,31 +2251,31 @@
         <f>INDEX(REASON_NO_BED,3)+INDEX(REASON_BEHAVIOR,3)+INDEX(REASON_SPECIAL_CARE,3)+INDEX(REASON_FINANCIAL,3)+INDEX(REASON_GUARDIANSHIP,3)+INDEX(REASON_PASARR,3)+INDEX(REASON_OTHER,3)</f>
         <v>184.0</v>
       </c>
-      <c r="M6" s="19">
+      <c r="M6" s="18">
         <f>INDEX(REASON_NO_BED,3)/INDEX(REASON_SUM,3)</f>
         <v>0.391304347826087</v>
       </c>
-      <c r="N6" s="19">
+      <c r="N6" s="18">
         <f>INDEX(REASON_BEHAVIOR,3)/INDEX(REASON_SUM,3)</f>
         <v>0.14673913043478262</v>
       </c>
-      <c r="O6" s="19">
+      <c r="O6" s="18">
         <f>INDEX(REASON_SPECIAL_CARE,3)/INDEX(REASON_SUM,3)</f>
         <v>0.11413043478260869</v>
       </c>
-      <c r="P6" s="19">
+      <c r="P6" s="18">
         <f>INDEX(REASON_FINANCIAL,3)/INDEX(REASON_SUM,3)</f>
         <v>0.17391304347826086</v>
       </c>
-      <c r="Q6" s="19">
+      <c r="Q6" s="18">
         <f>INDEX(REASON_GUARDIANSHIP,3)/INDEX(REASON_SUM,3)</f>
         <v>0.14130434782608695</v>
       </c>
-      <c r="R6" s="19">
+      <c r="R6" s="18">
         <f>INDEX(REASON_PASARR,3)/INDEX(REASON_SUM,3)</f>
         <v>0.0</v>
       </c>
-      <c r="S6" s="19">
+      <c r="S6" s="18">
         <f>INDEX(REASON_OTHER,3)/INDEX(REASON_SUM,3)</f>
         <v>0.03260869565217391</v>
       </c>
@@ -2302,7 +2301,7 @@
         <f>INDEX(WL_PATIENTS,4)*BENCH_DAYS</f>
         <v>63742.0</v>
       </c>
-      <c r="D7" s="18">
+      <c r="D7" s="16">
         <f>INDEX(DAYS_PER_PT,4)-BENCH_DAYS</f>
         <v>-1.4155501866900941</v>
       </c>
@@ -2318,7 +2317,7 @@
         <f>INDEX(WL_DAYS,4)-INDEX(EXCESS_DAYS,4)</f>
         <v>57297.0</v>
       </c>
-      <c r="H7" s="19">
+      <c r="H7" s="18">
         <f>INDEX(EXCESS_DAYS,4)/INDEX(WL_DAYS,4)</f>
         <v>0.0</v>
       </c>
@@ -2338,31 +2337,31 @@
         <f>INDEX(REASON_NO_BED,4)+INDEX(REASON_BEHAVIOR,4)+INDEX(REASON_SPECIAL_CARE,4)+INDEX(REASON_FINANCIAL,4)+INDEX(REASON_GUARDIANSHIP,4)+INDEX(REASON_PASARR,4)+INDEX(REASON_OTHER,4)</f>
         <v>144.0</v>
       </c>
-      <c r="M7" s="19">
+      <c r="M7" s="18">
         <f>INDEX(REASON_NO_BED,4)/INDEX(REASON_SUM,4)</f>
         <v>0.2847222222222222</v>
       </c>
-      <c r="N7" s="19">
+      <c r="N7" s="18">
         <f>INDEX(REASON_BEHAVIOR,4)/INDEX(REASON_SUM,4)</f>
         <v>0.16666666666666666</v>
       </c>
-      <c r="O7" s="19">
+      <c r="O7" s="18">
         <f>INDEX(REASON_SPECIAL_CARE,4)/INDEX(REASON_SUM,4)</f>
         <v>0.1527777777777778</v>
       </c>
-      <c r="P7" s="19">
+      <c r="P7" s="18">
         <f>INDEX(REASON_FINANCIAL,4)/INDEX(REASON_SUM,4)</f>
         <v>0.20833333333333334</v>
       </c>
-      <c r="Q7" s="19">
+      <c r="Q7" s="18">
         <f>INDEX(REASON_GUARDIANSHIP,4)/INDEX(REASON_SUM,4)</f>
         <v>0.10416666666666667</v>
       </c>
-      <c r="R7" s="19">
+      <c r="R7" s="18">
         <f>INDEX(REASON_PASARR,4)/INDEX(REASON_SUM,4)</f>
         <v>0.0</v>
       </c>
-      <c r="S7" s="19">
+      <c r="S7" s="18">
         <f>INDEX(REASON_OTHER,4)/INDEX(REASON_SUM,4)</f>
         <v>0.08333333333333333</v>
       </c>
@@ -2388,7 +2387,7 @@
         <f>INDEX(WL_PATIENTS,5)*BENCH_DAYS</f>
         <v>68978.0</v>
       </c>
-      <c r="D8" s="18">
+      <c r="D8" s="16">
         <f>INDEX(DAYS_PER_PT,5)-BENCH_DAYS</f>
         <v>-1.8120560178607672</v>
       </c>
@@ -2404,7 +2403,7 @@
         <f>INDEX(WL_DAYS,5)-INDEX(EXCESS_DAYS,5)</f>
         <v>60050.0</v>
       </c>
-      <c r="H8" s="19">
+      <c r="H8" s="18">
         <f>INDEX(EXCESS_DAYS,5)/INDEX(WL_DAYS,5)</f>
         <v>0.0</v>
       </c>
@@ -2424,31 +2423,31 @@
         <f>INDEX(REASON_NO_BED,5)+INDEX(REASON_BEHAVIOR,5)+INDEX(REASON_SPECIAL_CARE,5)+INDEX(REASON_FINANCIAL,5)+INDEX(REASON_GUARDIANSHIP,5)+INDEX(REASON_PASARR,5)+INDEX(REASON_OTHER,5)</f>
         <v>189.0</v>
       </c>
-      <c r="M8" s="19">
+      <c r="M8" s="18">
         <f>INDEX(REASON_NO_BED,5)/INDEX(REASON_SUM,5)</f>
         <v>0.26455026455026454</v>
       </c>
-      <c r="N8" s="19">
+      <c r="N8" s="18">
         <f>INDEX(REASON_BEHAVIOR,5)/INDEX(REASON_SUM,5)</f>
         <v>0.19047619047619047</v>
       </c>
-      <c r="O8" s="19">
+      <c r="O8" s="18">
         <f>INDEX(REASON_SPECIAL_CARE,5)/INDEX(REASON_SUM,5)</f>
         <v>0.1164021164021164</v>
       </c>
-      <c r="P8" s="19">
+      <c r="P8" s="18">
         <f>INDEX(REASON_FINANCIAL,5)/INDEX(REASON_SUM,5)</f>
         <v>0.2275132275132275</v>
       </c>
-      <c r="Q8" s="19">
+      <c r="Q8" s="18">
         <f>INDEX(REASON_GUARDIANSHIP,5)/INDEX(REASON_SUM,5)</f>
         <v>0.10582010582010581</v>
       </c>
-      <c r="R8" s="19">
+      <c r="R8" s="18">
         <f>INDEX(REASON_PASARR,5)/INDEX(REASON_SUM,5)</f>
         <v>0.0</v>
       </c>
-      <c r="S8" s="19">
+      <c r="S8" s="18">
         <f>INDEX(REASON_OTHER,5)/INDEX(REASON_SUM,5)</f>
         <v>0.09523809523809523</v>
       </c>
@@ -2474,7 +2473,7 @@
         <f>INDEX(WL_PATIENTS,6)*BENCH_DAYS</f>
         <v>51534.0</v>
       </c>
-      <c r="D9" s="18">
+      <c r="D9" s="16">
         <f>INDEX(DAYS_PER_PT,6)-BENCH_DAYS</f>
         <v>7.342298288508559</v>
       </c>
@@ -2490,7 +2489,7 @@
         <f>INDEX(WL_DAYS,6)-INDEX(EXCESS_DAYS,6)</f>
         <v>51534.0</v>
       </c>
-      <c r="H9" s="19">
+      <c r="H9" s="18">
         <f>INDEX(EXCESS_DAYS,6)/INDEX(WL_DAYS,6)</f>
         <v>0.3440256615878107</v>
       </c>
@@ -2510,31 +2509,31 @@
         <f>INDEX(REASON_NO_BED,6)+INDEX(REASON_BEHAVIOR,6)+INDEX(REASON_SPECIAL_CARE,6)+INDEX(REASON_FINANCIAL,6)+INDEX(REASON_GUARDIANSHIP,6)+INDEX(REASON_PASARR,6)+INDEX(REASON_OTHER,6)</f>
         <v>250.0</v>
       </c>
-      <c r="M9" s="19">
+      <c r="M9" s="18">
         <f>INDEX(REASON_NO_BED,6)/INDEX(REASON_SUM,6)</f>
         <v>0.228</v>
       </c>
-      <c r="N9" s="19">
+      <c r="N9" s="18">
         <f>INDEX(REASON_BEHAVIOR,6)/INDEX(REASON_SUM,6)</f>
         <v>0.14</v>
       </c>
-      <c r="O9" s="19">
+      <c r="O9" s="18">
         <f>INDEX(REASON_SPECIAL_CARE,6)/INDEX(REASON_SUM,6)</f>
         <v>0.156</v>
       </c>
-      <c r="P9" s="19">
+      <c r="P9" s="18">
         <f>INDEX(REASON_FINANCIAL,6)/INDEX(REASON_SUM,6)</f>
         <v>0.3</v>
       </c>
-      <c r="Q9" s="19">
+      <c r="Q9" s="18">
         <f>INDEX(REASON_GUARDIANSHIP,6)/INDEX(REASON_SUM,6)</f>
         <v>0.116</v>
       </c>
-      <c r="R9" s="19">
+      <c r="R9" s="18">
         <f>INDEX(REASON_PASARR,6)/INDEX(REASON_SUM,6)</f>
         <v>0.02</v>
       </c>
-      <c r="S9" s="19">
+      <c r="S9" s="18">
         <f>INDEX(REASON_OTHER,6)/INDEX(REASON_SUM,6)</f>
         <v>0.04</v>
       </c>
@@ -2560,7 +2559,7 @@
         <f>INDEX(WL_PATIENTS,7)*BENCH_DAYS</f>
         <v>50540.0</v>
       </c>
-      <c r="D10" s="18">
+      <c r="D10" s="16">
         <f>INDEX(DAYS_PER_PT,7)-BENCH_DAYS</f>
         <v>9.018559556786702</v>
       </c>
@@ -2576,7 +2575,7 @@
         <f>INDEX(WL_DAYS,7)-INDEX(EXCESS_DAYS,7)</f>
         <v>50540.0</v>
       </c>
-      <c r="H10" s="19">
+      <c r="H10" s="18">
         <f>INDEX(EXCESS_DAYS,7)/INDEX(WL_DAYS,7)</f>
         <v>0.3917951309914919</v>
       </c>
@@ -2596,31 +2595,31 @@
         <f>INDEX(REASON_NO_BED,7)+INDEX(REASON_BEHAVIOR,7)+INDEX(REASON_SPECIAL_CARE,7)+INDEX(REASON_FINANCIAL,7)+INDEX(REASON_GUARDIANSHIP,7)+INDEX(REASON_PASARR,7)+INDEX(REASON_OTHER,7)</f>
         <v>191.0</v>
       </c>
-      <c r="M10" s="19">
+      <c r="M10" s="18">
         <f>INDEX(REASON_NO_BED,7)/INDEX(REASON_SUM,7)</f>
         <v>0.2198952879581152</v>
       </c>
-      <c r="N10" s="19">
+      <c r="N10" s="18">
         <f>INDEX(REASON_BEHAVIOR,7)/INDEX(REASON_SUM,7)</f>
         <v>0.2513089005235602</v>
       </c>
-      <c r="O10" s="19">
+      <c r="O10" s="18">
         <f>INDEX(REASON_SPECIAL_CARE,7)/INDEX(REASON_SUM,7)</f>
         <v>0.13612565445026178</v>
       </c>
-      <c r="P10" s="19">
+      <c r="P10" s="18">
         <f>INDEX(REASON_FINANCIAL,7)/INDEX(REASON_SUM,7)</f>
         <v>0.2356020942408377</v>
       </c>
-      <c r="Q10" s="19">
+      <c r="Q10" s="18">
         <f>INDEX(REASON_GUARDIANSHIP,7)/INDEX(REASON_SUM,7)</f>
         <v>0.14659685863874344</v>
       </c>
-      <c r="R10" s="19">
+      <c r="R10" s="18">
         <f>INDEX(REASON_PASARR,7)/INDEX(REASON_SUM,7)</f>
         <v>0.005235602094240838</v>
       </c>
-      <c r="S10" s="19">
+      <c r="S10" s="18">
         <f>INDEX(REASON_OTHER,7)/INDEX(REASON_SUM,7)</f>
         <v>0.005235602094240838</v>
       </c>
@@ -2646,7 +2645,7 @@
         <f>INDEX(WL_PATIENTS,8)*BENCH_DAYS</f>
         <v>43722.0</v>
       </c>
-      <c r="D11" s="18">
+      <c r="D11" s="16">
         <f>INDEX(DAYS_PER_PT,8)-BENCH_DAYS</f>
         <v>5.492795389048993</v>
       </c>
@@ -2662,7 +2661,7 @@
         <f>INDEX(WL_DAYS,8)-INDEX(EXCESS_DAYS,8)</f>
         <v>43722.0</v>
       </c>
-      <c r="H11" s="19">
+      <c r="H11" s="18">
         <f>INDEX(EXCESS_DAYS,8)/INDEX(WL_DAYS,8)</f>
         <v>0.281785925487877</v>
       </c>
@@ -2682,31 +2681,31 @@
         <f>INDEX(REASON_NO_BED,8)+INDEX(REASON_BEHAVIOR,8)+INDEX(REASON_SPECIAL_CARE,8)+INDEX(REASON_FINANCIAL,8)+INDEX(REASON_GUARDIANSHIP,8)+INDEX(REASON_PASARR,8)+INDEX(REASON_OTHER,8)</f>
         <v>173.0</v>
       </c>
-      <c r="M11" s="19">
+      <c r="M11" s="18">
         <f>INDEX(REASON_NO_BED,8)/INDEX(REASON_SUM,8)</f>
         <v>0.1791907514450867</v>
       </c>
-      <c r="N11" s="19">
+      <c r="N11" s="18">
         <f>INDEX(REASON_BEHAVIOR,8)/INDEX(REASON_SUM,8)</f>
         <v>0.1676300578034682</v>
       </c>
-      <c r="O11" s="19">
+      <c r="O11" s="18">
         <f>INDEX(REASON_SPECIAL_CARE,8)/INDEX(REASON_SUM,8)</f>
         <v>0.10404624277456648</v>
       </c>
-      <c r="P11" s="19">
+      <c r="P11" s="18">
         <f>INDEX(REASON_FINANCIAL,8)/INDEX(REASON_SUM,8)</f>
         <v>0.3468208092485549</v>
       </c>
-      <c r="Q11" s="19">
+      <c r="Q11" s="18">
         <f>INDEX(REASON_GUARDIANSHIP,8)/INDEX(REASON_SUM,8)</f>
         <v>0.1791907514450867</v>
       </c>
-      <c r="R11" s="19">
+      <c r="R11" s="18">
         <f>INDEX(REASON_PASARR,8)/INDEX(REASON_SUM,8)</f>
         <v>0.0</v>
       </c>
-      <c r="S11" s="19">
+      <c r="S11" s="18">
         <f>INDEX(REASON_OTHER,8)/INDEX(REASON_SUM,8)</f>
         <v>0.023121387283236993</v>
       </c>
@@ -2832,7 +2831,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="20" t="inlineStr">
+      <c r="A4" s="19" t="inlineStr">
         <is>
           <t>Excess days</t>
         </is>
@@ -2856,7 +2855,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>Waitlisted rate, January</t>
         </is>
@@ -2866,17 +2865,17 @@
           <t>USD per day</t>
         </is>
       </c>
-      <c r="C5" s="21">
+      <c r="C5" s="20">
         <f>INDEX(WL_RATE_JAN,MATCH(2023,YEAR,0))</f>
         <v>283.6</v>
       </c>
-      <c r="D5" s="21">
+      <c r="D5" s="20">
         <f>INDEX(WL_RATE_JAN,MATCH(2024,YEAR,0))</f>
         <v>464.97</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="20" t="inlineStr">
+      <c r="A6" s="19" t="inlineStr">
         <is>
           <t>Waitlisted rate, July</t>
         </is>
@@ -2886,17 +2885,17 @@
           <t>USD per day</t>
         </is>
       </c>
-      <c r="C6" s="21">
+      <c r="C6" s="20">
         <f>INDEX(WL_RATE_JUL,MATCH(2023,YEAR,0))</f>
         <v>302.89</v>
       </c>
-      <c r="D6" s="21">
+      <c r="D6" s="20">
         <f>INDEX(WL_RATE_JUL,MATCH(2024,YEAR,0))</f>
         <v>455.59</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="20" t="inlineStr">
+    <row r="7" ht="31" customHeight="1">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>Average waitlisted rate (WL_RATE_AVG); Now = WL_RATE_2026</t>
         </is>
@@ -2906,21 +2905,21 @@
           <t>USD per day</t>
         </is>
       </c>
-      <c r="C7" s="22">
+      <c r="C7" s="20">
         <f>(INDEX(WL_RATE_JAN,MATCH(2023,YEAR,0))+INDEX(WL_RATE_JUL,MATCH(2023,YEAR,0)))/2</f>
         <v>293.245</v>
       </c>
-      <c r="D7" s="22">
+      <c r="D7" s="20">
         <f>(INDEX(WL_RATE_JAN,MATCH(2024,YEAR,0))+INDEX(WL_RATE_JUL,MATCH(2024,YEAR,0)))/2</f>
         <v>460.28</v>
       </c>
-      <c r="E7" s="22">
+      <c r="E7" s="20">
         <f>WL_RATE_2026</f>
         <v>486.76</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>Net cost per day, low (NET_COST_LO)</t>
         </is>
@@ -2930,21 +2929,21 @@
           <t>USD per day</t>
         </is>
       </c>
-      <c r="C8" s="21">
+      <c r="C8" s="20">
         <f>AVOID_COST_LO-INDEX(WL_RATE_AVG,1)</f>
         <v>256.755</v>
       </c>
-      <c r="D8" s="21">
+      <c r="D8" s="20">
         <f>AVOID_COST_LO-INDEX(WL_RATE_AVG,2)</f>
         <v>89.72000000000003</v>
       </c>
-      <c r="E8" s="21">
+      <c r="E8" s="20">
         <f>AVOID_COST_LO-WL_RATE_2026</f>
         <v>63.24000000000001</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>Net cost per day, high (NET_COST_HI)</t>
         </is>
@@ -2954,21 +2953,21 @@
           <t>USD per day</t>
         </is>
       </c>
-      <c r="C9" s="21">
+      <c r="C9" s="20">
         <f>AVOID_COST_HI-INDEX(WL_RATE_AVG,1)</f>
         <v>1176.755</v>
       </c>
-      <c r="D9" s="21">
+      <c r="D9" s="20">
         <f>AVOID_COST_HI-INDEX(WL_RATE_AVG,2)</f>
         <v>1009.72</v>
       </c>
-      <c r="E9" s="21">
+      <c r="E9" s="20">
         <f>AVOID_COST_HI-WL_RATE_2026</f>
         <v>983.24</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="20" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>Cost of excess days, low (EXCESS_COST_LO)</t>
         </is>
@@ -2978,21 +2977,21 @@
           <t>USD per year</t>
         </is>
       </c>
-      <c r="C10" s="23">
+      <c r="C10" s="21">
         <f>INDEX(EXCESS_DAYS,MATCH(2023,YEAR,0))*INDEX(NET_COST_LO,1)</f>
         <v>8359172.535</v>
       </c>
-      <c r="D10" s="23">
+      <c r="D10" s="21">
         <f>INDEX(EXCESS_DAYS,MATCH(2024,YEAR,0))*INDEX(NET_COST_LO,2)</f>
         <v>1539056.8800000004</v>
       </c>
-      <c r="E10" s="23">
+      <c r="E10" s="21">
         <f>INDEX(EXCESS_DAYS,MATCH(2024,YEAR,0))*NET_COST_LO_NOW</f>
         <v>1084818.9600000002</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="20" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>Cost of excess days, high (EXCESS_COST_HI)</t>
         </is>
@@ -3002,21 +3001,21 @@
           <t>USD per year</t>
         </is>
       </c>
-      <c r="C11" s="23">
+      <c r="C11" s="21">
         <f>INDEX(EXCESS_DAYS,MATCH(2023,YEAR,0))*INDEX(NET_COST_HI,1)</f>
         <v>38311612.535000004</v>
       </c>
-      <c r="D11" s="23">
+      <c r="D11" s="21">
         <f>INDEX(EXCESS_DAYS,MATCH(2024,YEAR,0))*INDEX(NET_COST_HI,2)</f>
         <v>17320736.88</v>
       </c>
-      <c r="E11" s="23">
+      <c r="E11" s="21">
         <f>INDEX(EXCESS_DAYS,MATCH(2024,YEAR,0))*NET_COST_HI_NOW</f>
         <v>16866498.96</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="20" t="inlineStr">
+    <row r="12" ht="31" customHeight="1">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>Nursing-facility share of Dec 31 waitlist (NF_SHARE_DEC31), reported beside the result only</t>
         </is>
@@ -3026,17 +3025,17 @@
           <t>share</t>
         </is>
       </c>
-      <c r="C12" s="19">
+      <c r="C12" s="18">
         <f>INDEX(DEC31_NF,MATCH(2023,YEAR,0))/INDEX(DEC31_TOTAL,MATCH(2023,YEAR,0))</f>
         <v>0.8219895287958116</v>
       </c>
-      <c r="D12" s="19">
+      <c r="D12" s="18">
         <f>INDEX(DEC31_NF,MATCH(2024,YEAR,0))/INDEX(DEC31_TOTAL,MATCH(2024,YEAR,0))</f>
         <v>0.6936416184971098</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="20" t="inlineStr">
+    <row r="14" ht="31" customHeight="1">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>Change in waitlist days, 2023 to 2024 (WL_DAYS_CHANGE_2024)</t>
         </is>
@@ -3046,7 +3045,7 @@
           <t>share</t>
         </is>
       </c>
-      <c r="C14" s="19">
+      <c r="C14" s="18">
         <f>INDEX(WL_DAYS,MATCH(2024,YEAR,0))/INDEX(WL_DAYS,MATCH(2023,YEAR,0))-1</f>
         <v>-0.26741037582584204</v>
       </c>
@@ -3062,7 +3061,7 @@
           <t>USD per day</t>
         </is>
       </c>
-      <c r="C15" s="21">
+      <c r="C15" s="20">
         <f>WL_RATE_LEAHI_2026</f>
         <v>480.19</v>
       </c>
@@ -3093,7 +3092,7 @@
   <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="82" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
@@ -3130,7 +3129,7 @@
           <t>Financial share, Dec 31 2020</t>
         </is>
       </c>
-      <c r="B4" s="24">
+      <c r="B4" s="18">
         <f>INDEX(SHARE_FINANCIAL,MATCH(2020,YEAR,0))</f>
         <v>0.20833333333333334</v>
       </c>
@@ -3146,7 +3145,7 @@
           <t>Financial share, Dec 31 2021</t>
         </is>
       </c>
-      <c r="B5" s="24">
+      <c r="B5" s="18">
         <f>INDEX(SHARE_FINANCIAL,MATCH(2021,YEAR,0))</f>
         <v>0.2275132275132275</v>
       </c>
@@ -3162,7 +3161,7 @@
           <t>Drop, 2020 to 2021 (T1_DROP_2021; negative = rise)</t>
         </is>
       </c>
-      <c r="B6" s="24">
+      <c r="B6" s="18">
         <f>INDEX(SHARE_FINANCIAL,MATCH(2020,YEAR,0))-INDEX(SHARE_FINANCIAL,MATCH(2021,YEAR,0))</f>
         <v>-0.019179894179894158</v>
       </c>
@@ -3194,7 +3193,7 @@
           <t>Financial share, Dec 31 2023</t>
         </is>
       </c>
-      <c r="B8" s="24">
+      <c r="B8" s="18">
         <f>INDEX(SHARE_FINANCIAL,MATCH(2023,YEAR,0))</f>
         <v>0.2356020942408377</v>
       </c>
@@ -3205,7 +3204,7 @@
           <t>Financial share, Dec 31 2024</t>
         </is>
       </c>
-      <c r="B9" s="24">
+      <c r="B9" s="18">
         <f>INDEX(SHARE_FINANCIAL,MATCH(2024,YEAR,0))</f>
         <v>0.3468208092485549</v>
       </c>
@@ -3216,7 +3215,7 @@
           <t>Drop, 2023 to 2024 (T1_DROP_2024; negative = rise)</t>
         </is>
       </c>
-      <c r="B10" s="24">
+      <c r="B10" s="18">
         <f>INDEX(SHARE_FINANCIAL,MATCH(2023,YEAR,0))-INDEX(SHARE_FINANCIAL,MATCH(2024,YEAR,0))</f>
         <v>-0.11121871500771721</v>
       </c>
@@ -3281,7 +3280,7 @@
           <t>Least-squares slope of days per patient, 2017 to 2023 (T2_SLOPE)</t>
         </is>
       </c>
-      <c r="B15" s="18">
+      <c r="B15" s="16">
         <f>SLOPE(INDEX(DAYS_PER_PT,1):INDEX(DAYS_PER_PT,7),INDEX(YEAR,1):INDEX(YEAR,7))</f>
         <v>1.8814212714379457</v>
       </c>
@@ -3633,11 +3632,11 @@
         <f>INDEX(CTY_DAYS,1,2)/INDEX(CTY_PATIENTS,1,2)</f>
         <v>27.74965612104539</v>
       </c>
-      <c r="D4" s="19">
+      <c r="D4" s="18">
         <f>INDEX(CTY_DAYS,1,1)/INDEX(WL_DAYS,MATCH(2023,YEAR,0))</f>
         <v>0.27933619745598515</v>
       </c>
-      <c r="E4" s="19">
+      <c r="E4" s="18">
         <f>INDEX(CTY_DAYS,1,2)/INDEX(WL_DAYS,MATCH(2024,YEAR,0))</f>
         <v>0.33139496681779357</v>
       </c>
@@ -3655,11 +3654,11 @@
         <f>INDEX(CTY_DAYS,2,2)/INDEX(CTY_PATIENTS,2,2)</f>
         <v>13.835270338554826</v>
       </c>
-      <c r="D5" s="19">
+      <c r="D5" s="18">
         <f>INDEX(CTY_DAYS,2,1)/INDEX(WL_DAYS,MATCH(2023,YEAR,0))</f>
         <v>0.4853003116839356</v>
       </c>
-      <c r="E5" s="19">
+      <c r="E5" s="18">
         <f>INDEX(CTY_DAYS,2,2)/INDEX(WL_DAYS,MATCH(2024,YEAR,0))</f>
         <v>0.4497667389447401</v>
       </c>
@@ -3677,11 +3676,11 @@
         <f>INDEX(CTY_DAYS,3,2)/INDEX(CTY_PATIENTS,3,2)</f>
         <v>30.109375</v>
       </c>
-      <c r="D6" s="19">
+      <c r="D6" s="18">
         <f>INDEX(CTY_DAYS,3,1)/INDEX(WL_DAYS,MATCH(2023,YEAR,0))</f>
         <v>0.02069870151750364</v>
       </c>
-      <c r="E6" s="19">
+      <c r="E6" s="18">
         <f>INDEX(CTY_DAYS,3,2)/INDEX(WL_DAYS,MATCH(2024,YEAR,0))</f>
         <v>0.031654510808857346</v>
       </c>
@@ -3699,11 +3698,11 @@
         <f>INDEX(CTY_DAYS,4,2)/INDEX(CTY_PATIENTS,4,2)</f>
         <v>32.28045325779037</v>
       </c>
-      <c r="D7" s="19">
+      <c r="D7" s="18">
         <f>INDEX(CTY_DAYS,4,1)/INDEX(WL_DAYS,MATCH(2023,YEAR,0))</f>
         <v>0.21466478934257555</v>
       </c>
-      <c r="E7" s="19">
+      <c r="E7" s="18">
         <f>INDEX(CTY_DAYS,4,2)/INDEX(WL_DAYS,MATCH(2024,YEAR,0))</f>
         <v>0.18718378342860897</v>
       </c>
@@ -3714,11 +3713,11 @@
           <t>Total share</t>
         </is>
       </c>
-      <c r="D8" s="19">
+      <c r="D8" s="18">
         <f>INDEX(CTY_DAY_SHARE,1,1)+INDEX(CTY_DAY_SHARE,2,1)+INDEX(CTY_DAY_SHARE,3,1)+INDEX(CTY_DAY_SHARE,4,1)</f>
         <v>1.0</v>
       </c>
-      <c r="E8" s="19">
+      <c r="E8" s="18">
         <f>INDEX(CTY_DAY_SHARE,1,2)+INDEX(CTY_DAY_SHARE,2,2)+INDEX(CTY_DAY_SHARE,3,2)+INDEX(CTY_DAY_SHARE,4,2)</f>
         <v>1.0</v>
       </c>
@@ -3744,7 +3743,7 @@
   <dimension ref="A1:I86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
@@ -3752,7 +3751,7 @@
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3801,11 +3800,11 @@
         <f>INDEX(YEAR,1)</f>
         <v>2017</v>
       </c>
-      <c r="B5" s="25">
+      <c r="B5" s="22">
         <f>DATE(INDEX(YEAR,1),7,1)</f>
         <v>42917</v>
       </c>
-      <c r="C5" s="18">
+      <c r="C5" s="16">
         <f>INDEX(DAYS_PER_PT,1)</f>
         <v>9.935348310974625</v>
       </c>
@@ -3823,11 +3822,11 @@
         <f>INDEX(YEAR,2)</f>
         <v>2018</v>
       </c>
-      <c r="B6" s="25">
+      <c r="B6" s="22">
         <f>DATE(INDEX(YEAR,2),7,1)</f>
         <v>43282</v>
       </c>
-      <c r="C6" s="18">
+      <c r="C6" s="16">
         <f>INDEX(DAYS_PER_PT,2)</f>
         <v>12.484132980732905</v>
       </c>
@@ -3845,11 +3844,11 @@
         <f>INDEX(YEAR,3)</f>
         <v>2019</v>
       </c>
-      <c r="B7" s="25">
+      <c r="B7" s="22">
         <f>DATE(INDEX(YEAR,3),7,1)</f>
         <v>43647</v>
       </c>
-      <c r="C7" s="18">
+      <c r="C7" s="16">
         <f>INDEX(DAYS_PER_PT,3)</f>
         <v>16.4741127348643</v>
       </c>
@@ -3867,11 +3866,11 @@
         <f>INDEX(YEAR,4)</f>
         <v>2020</v>
       </c>
-      <c r="B8" s="25">
+      <c r="B8" s="22">
         <f>DATE(INDEX(YEAR,4),7,1)</f>
         <v>44013</v>
       </c>
-      <c r="C8" s="18">
+      <c r="C8" s="16">
         <f>INDEX(DAYS_PER_PT,4)</f>
         <v>12.584449813309906</v>
       </c>
@@ -3889,11 +3888,11 @@
         <f>INDEX(YEAR,5)</f>
         <v>2021</v>
       </c>
-      <c r="B9" s="25">
+      <c r="B9" s="22">
         <f>DATE(INDEX(YEAR,5),7,1)</f>
         <v>44378</v>
       </c>
-      <c r="C9" s="18">
+      <c r="C9" s="16">
         <f>INDEX(DAYS_PER_PT,5)</f>
         <v>12.187943982139233</v>
       </c>
@@ -3911,11 +3910,11 @@
         <f>INDEX(YEAR,6)</f>
         <v>2022</v>
       </c>
-      <c r="B10" s="25">
+      <c r="B10" s="22">
         <f>DATE(INDEX(YEAR,6),7,1)</f>
         <v>44743</v>
       </c>
-      <c r="C10" s="18">
+      <c r="C10" s="16">
         <f>INDEX(DAYS_PER_PT,6)</f>
         <v>21.34229828850856</v>
       </c>
@@ -3933,11 +3932,11 @@
         <f>INDEX(YEAR,7)</f>
         <v>2023</v>
       </c>
-      <c r="B11" s="25">
+      <c r="B11" s="22">
         <f>DATE(INDEX(YEAR,7),7,1)</f>
         <v>45108</v>
       </c>
-      <c r="C11" s="18">
+      <c r="C11" s="16">
         <f>INDEX(DAYS_PER_PT,7)</f>
         <v>23.018559556786702</v>
       </c>
@@ -3955,11 +3954,11 @@
         <f>INDEX(YEAR,8)</f>
         <v>2024</v>
       </c>
-      <c r="B12" s="25">
+      <c r="B12" s="22">
         <f>DATE(INDEX(YEAR,8),7,1)</f>
         <v>45474</v>
       </c>
-      <c r="C12" s="18">
+      <c r="C12" s="16">
         <f>INDEX(DAYS_PER_PT,8)</f>
         <v>19.492795389048993</v>
       </c>
@@ -3997,7 +3996,7 @@
           <t>12% adjustment for private homes</t>
         </is>
       </c>
-      <c r="B16" s="25">
+      <c r="B16" s="22">
         <f>DATE_ADJ_2021</f>
         <v>44209</v>
       </c>
@@ -4008,7 +4007,7 @@
           <t>Rate reset</t>
         </is>
       </c>
-      <c r="B17" s="25">
+      <c r="B17" s="22">
         <f>DATE_RESET_2024</f>
         <v>45292</v>
       </c>
@@ -4072,31 +4071,31 @@
         <f>INDEX(YEAR,1)</f>
         <v>2017</v>
       </c>
-      <c r="B21" s="19">
+      <c r="B21" s="18">
         <f>INDEX(SHARE_NO_BED,1)</f>
         <v>0.325</v>
       </c>
-      <c r="C21" s="19">
+      <c r="C21" s="18">
         <f>INDEX(SHARE_BEHAVIOR,1)</f>
         <v>0.13333333333333333</v>
       </c>
-      <c r="D21" s="19">
+      <c r="D21" s="18">
         <f>INDEX(SHARE_SPECIAL_CARE,1)</f>
         <v>0.19166666666666668</v>
       </c>
-      <c r="E21" s="19">
+      <c r="E21" s="18">
         <f>INDEX(SHARE_FINANCIAL,1)</f>
         <v>0.15</v>
       </c>
-      <c r="F21" s="19">
+      <c r="F21" s="18">
         <f>INDEX(SHARE_GUARDIANSHIP,1)</f>
         <v>0.09166666666666666</v>
       </c>
-      <c r="G21" s="19">
+      <c r="G21" s="18">
         <f>INDEX(SHARE_PASARR,1)</f>
         <v>0.016666666666666666</v>
       </c>
-      <c r="H21" s="19">
+      <c r="H21" s="18">
         <f>INDEX(SHARE_OTHER,1)</f>
         <v>0.09166666666666666</v>
       </c>
@@ -4110,31 +4109,31 @@
         <f>INDEX(YEAR,2)</f>
         <v>2018</v>
       </c>
-      <c r="B22" s="19">
+      <c r="B22" s="18">
         <f>INDEX(SHARE_NO_BED,2)</f>
         <v>0.3333333333333333</v>
       </c>
-      <c r="C22" s="19">
+      <c r="C22" s="18">
         <f>INDEX(SHARE_BEHAVIOR,2)</f>
         <v>0.1695906432748538</v>
       </c>
-      <c r="D22" s="19">
+      <c r="D22" s="18">
         <f>INDEX(SHARE_SPECIAL_CARE,2)</f>
         <v>0.09941520467836257</v>
       </c>
-      <c r="E22" s="19">
+      <c r="E22" s="18">
         <f>INDEX(SHARE_FINANCIAL,2)</f>
         <v>0.18128654970760233</v>
       </c>
-      <c r="F22" s="19">
+      <c r="F22" s="18">
         <f>INDEX(SHARE_GUARDIANSHIP,2)</f>
         <v>0.10526315789473684</v>
       </c>
-      <c r="G22" s="19">
+      <c r="G22" s="18">
         <f>INDEX(SHARE_PASARR,2)</f>
         <v>0.011695906432748537</v>
       </c>
-      <c r="H22" s="19">
+      <c r="H22" s="18">
         <f>INDEX(SHARE_OTHER,2)</f>
         <v>0.09941520467836257</v>
       </c>
@@ -4148,31 +4147,31 @@
         <f>INDEX(YEAR,3)</f>
         <v>2019</v>
       </c>
-      <c r="B23" s="19">
+      <c r="B23" s="18">
         <f>INDEX(SHARE_NO_BED,3)</f>
         <v>0.391304347826087</v>
       </c>
-      <c r="C23" s="19">
+      <c r="C23" s="18">
         <f>INDEX(SHARE_BEHAVIOR,3)</f>
         <v>0.14673913043478262</v>
       </c>
-      <c r="D23" s="19">
+      <c r="D23" s="18">
         <f>INDEX(SHARE_SPECIAL_CARE,3)</f>
         <v>0.11413043478260869</v>
       </c>
-      <c r="E23" s="19">
+      <c r="E23" s="18">
         <f>INDEX(SHARE_FINANCIAL,3)</f>
         <v>0.17391304347826086</v>
       </c>
-      <c r="F23" s="19">
+      <c r="F23" s="18">
         <f>INDEX(SHARE_GUARDIANSHIP,3)</f>
         <v>0.14130434782608695</v>
       </c>
-      <c r="G23" s="19">
+      <c r="G23" s="18">
         <f>INDEX(SHARE_PASARR,3)</f>
         <v>0.0</v>
       </c>
-      <c r="H23" s="19">
+      <c r="H23" s="18">
         <f>INDEX(SHARE_OTHER,3)</f>
         <v>0.03260869565217391</v>
       </c>
@@ -4186,31 +4185,31 @@
         <f>INDEX(YEAR,4)</f>
         <v>2020</v>
       </c>
-      <c r="B24" s="19">
+      <c r="B24" s="18">
         <f>INDEX(SHARE_NO_BED,4)</f>
         <v>0.2847222222222222</v>
       </c>
-      <c r="C24" s="19">
+      <c r="C24" s="18">
         <f>INDEX(SHARE_BEHAVIOR,4)</f>
         <v>0.16666666666666666</v>
       </c>
-      <c r="D24" s="19">
+      <c r="D24" s="18">
         <f>INDEX(SHARE_SPECIAL_CARE,4)</f>
         <v>0.1527777777777778</v>
       </c>
-      <c r="E24" s="19">
+      <c r="E24" s="18">
         <f>INDEX(SHARE_FINANCIAL,4)</f>
         <v>0.20833333333333334</v>
       </c>
-      <c r="F24" s="19">
+      <c r="F24" s="18">
         <f>INDEX(SHARE_GUARDIANSHIP,4)</f>
         <v>0.10416666666666667</v>
       </c>
-      <c r="G24" s="19">
+      <c r="G24" s="18">
         <f>INDEX(SHARE_PASARR,4)</f>
         <v>0.0</v>
       </c>
-      <c r="H24" s="19">
+      <c r="H24" s="18">
         <f>INDEX(SHARE_OTHER,4)</f>
         <v>0.08333333333333333</v>
       </c>
@@ -4224,31 +4223,31 @@
         <f>INDEX(YEAR,5)</f>
         <v>2021</v>
       </c>
-      <c r="B25" s="19">
+      <c r="B25" s="18">
         <f>INDEX(SHARE_NO_BED,5)</f>
         <v>0.26455026455026454</v>
       </c>
-      <c r="C25" s="19">
+      <c r="C25" s="18">
         <f>INDEX(SHARE_BEHAVIOR,5)</f>
         <v>0.19047619047619047</v>
       </c>
-      <c r="D25" s="19">
+      <c r="D25" s="18">
         <f>INDEX(SHARE_SPECIAL_CARE,5)</f>
         <v>0.1164021164021164</v>
       </c>
-      <c r="E25" s="19">
+      <c r="E25" s="18">
         <f>INDEX(SHARE_FINANCIAL,5)</f>
         <v>0.2275132275132275</v>
       </c>
-      <c r="F25" s="19">
+      <c r="F25" s="18">
         <f>INDEX(SHARE_GUARDIANSHIP,5)</f>
         <v>0.10582010582010581</v>
       </c>
-      <c r="G25" s="19">
+      <c r="G25" s="18">
         <f>INDEX(SHARE_PASARR,5)</f>
         <v>0.0</v>
       </c>
-      <c r="H25" s="19">
+      <c r="H25" s="18">
         <f>INDEX(SHARE_OTHER,5)</f>
         <v>0.09523809523809523</v>
       </c>
@@ -4262,31 +4261,31 @@
         <f>INDEX(YEAR,6)</f>
         <v>2022</v>
       </c>
-      <c r="B26" s="19">
+      <c r="B26" s="18">
         <f>INDEX(SHARE_NO_BED,6)</f>
         <v>0.228</v>
       </c>
-      <c r="C26" s="19">
+      <c r="C26" s="18">
         <f>INDEX(SHARE_BEHAVIOR,6)</f>
         <v>0.14</v>
       </c>
-      <c r="D26" s="19">
+      <c r="D26" s="18">
         <f>INDEX(SHARE_SPECIAL_CARE,6)</f>
         <v>0.156</v>
       </c>
-      <c r="E26" s="19">
+      <c r="E26" s="18">
         <f>INDEX(SHARE_FINANCIAL,6)</f>
         <v>0.3</v>
       </c>
-      <c r="F26" s="19">
+      <c r="F26" s="18">
         <f>INDEX(SHARE_GUARDIANSHIP,6)</f>
         <v>0.116</v>
       </c>
-      <c r="G26" s="19">
+      <c r="G26" s="18">
         <f>INDEX(SHARE_PASARR,6)</f>
         <v>0.02</v>
       </c>
-      <c r="H26" s="19">
+      <c r="H26" s="18">
         <f>INDEX(SHARE_OTHER,6)</f>
         <v>0.04</v>
       </c>
@@ -4300,31 +4299,31 @@
         <f>INDEX(YEAR,7)</f>
         <v>2023</v>
       </c>
-      <c r="B27" s="19">
+      <c r="B27" s="18">
         <f>INDEX(SHARE_NO_BED,7)</f>
         <v>0.2198952879581152</v>
       </c>
-      <c r="C27" s="19">
+      <c r="C27" s="18">
         <f>INDEX(SHARE_BEHAVIOR,7)</f>
         <v>0.2513089005235602</v>
       </c>
-      <c r="D27" s="19">
+      <c r="D27" s="18">
         <f>INDEX(SHARE_SPECIAL_CARE,7)</f>
         <v>0.13612565445026178</v>
       </c>
-      <c r="E27" s="19">
+      <c r="E27" s="18">
         <f>INDEX(SHARE_FINANCIAL,7)</f>
         <v>0.2356020942408377</v>
       </c>
-      <c r="F27" s="19">
+      <c r="F27" s="18">
         <f>INDEX(SHARE_GUARDIANSHIP,7)</f>
         <v>0.14659685863874344</v>
       </c>
-      <c r="G27" s="19">
+      <c r="G27" s="18">
         <f>INDEX(SHARE_PASARR,7)</f>
         <v>0.005235602094240838</v>
       </c>
-      <c r="H27" s="19">
+      <c r="H27" s="18">
         <f>INDEX(SHARE_OTHER,7)</f>
         <v>0.005235602094240838</v>
       </c>
@@ -4338,31 +4337,31 @@
         <f>INDEX(YEAR,8)</f>
         <v>2024</v>
       </c>
-      <c r="B28" s="19">
+      <c r="B28" s="18">
         <f>INDEX(SHARE_NO_BED,8)</f>
         <v>0.1791907514450867</v>
       </c>
-      <c r="C28" s="19">
+      <c r="C28" s="18">
         <f>INDEX(SHARE_BEHAVIOR,8)</f>
         <v>0.1676300578034682</v>
       </c>
-      <c r="D28" s="19">
+      <c r="D28" s="18">
         <f>INDEX(SHARE_SPECIAL_CARE,8)</f>
         <v>0.10404624277456648</v>
       </c>
-      <c r="E28" s="19">
+      <c r="E28" s="18">
         <f>INDEX(SHARE_FINANCIAL,8)</f>
         <v>0.3468208092485549</v>
       </c>
-      <c r="F28" s="19">
+      <c r="F28" s="18">
         <f>INDEX(SHARE_GUARDIANSHIP,8)</f>
         <v>0.1791907514450867</v>
       </c>
-      <c r="G28" s="19">
+      <c r="G28" s="18">
         <f>INDEX(SHARE_PASARR,8)</f>
         <v>0.0</v>
       </c>
-      <c r="H28" s="19">
+      <c r="H28" s="18">
         <f>INDEX(SHARE_OTHER,8)</f>
         <v>0.023121387283236993</v>
       </c>
@@ -4401,11 +4400,11 @@
           <t>Across the 12% adjustment</t>
         </is>
       </c>
-      <c r="B32" s="26">
+      <c r="B32" s="23">
         <f>YEAR(DATE_ADJ_2021)-1</f>
         <v>2020.0</v>
       </c>
-      <c r="C32" s="26">
+      <c r="C32" s="23">
         <f>YEAR(DATE_ADJ_2021)</f>
         <v>2021</v>
       </c>
@@ -4416,11 +4415,11 @@
           <t>Across the reset</t>
         </is>
       </c>
-      <c r="B33" s="26">
+      <c r="B33" s="23">
         <f>YEAR(DATE_RESET_2024)-1</f>
         <v>2023.0</v>
       </c>
-      <c r="C33" s="26">
+      <c r="C33" s="23">
         <f>YEAR(DATE_RESET_2024)</f>
         <v>2024</v>
       </c>
@@ -4454,7 +4453,7 @@
         <f>DATE(2016,1,1)</f>
         <v>42370</v>
       </c>
-      <c r="B37" s="21">
+      <c r="B37" s="20">
         <f>IF(ISNA(MATCH(A37,RATE_DATE,0)),"",IF(INDEX(NF_RATE_MEDIAN,MATCH(A37,RATE_DATE,0))="","",INDEX(NF_RATE_MEDIAN,MATCH(A37,RATE_DATE,0))))</f>
         <v>246.97</v>
       </c>
@@ -4468,7 +4467,7 @@
         <f>DATE(2016,7,1)</f>
         <v>42552</v>
       </c>
-      <c r="B38" s="21">
+      <c r="B38" s="20">
         <f>IF(ISNA(MATCH(A38,RATE_DATE,0)),"",IF(INDEX(NF_RATE_MEDIAN,MATCH(A38,RATE_DATE,0))="","",INDEX(NF_RATE_MEDIAN,MATCH(A38,RATE_DATE,0))))</f>
         <v>252.4</v>
       </c>
@@ -4482,7 +4481,7 @@
         <f>DATE(2017,1,1)</f>
         <v>42736</v>
       </c>
-      <c r="B39" s="21">
+      <c r="B39" s="20">
         <f>IF(ISNA(MATCH(A39,RATE_DATE,0)),"",IF(INDEX(NF_RATE_MEDIAN,MATCH(A39,RATE_DATE,0))="","",INDEX(NF_RATE_MEDIAN,MATCH(A39,RATE_DATE,0))))</f>
         <v>251.93</v>
       </c>
@@ -4496,7 +4495,7 @@
         <f>DATE(2017,7,1)</f>
         <v>42917</v>
       </c>
-      <c r="B40" s="21">
+      <c r="B40" s="20">
         <f>IF(ISNA(MATCH(A40,RATE_DATE,0)),"",IF(INDEX(NF_RATE_MEDIAN,MATCH(A40,RATE_DATE,0))="","",INDEX(NF_RATE_MEDIAN,MATCH(A40,RATE_DATE,0))))</f>
         <v>261.45</v>
       </c>
@@ -4510,7 +4509,7 @@
         <f>DATE(2018,1,1)</f>
         <v>43101</v>
       </c>
-      <c r="B41" s="21" t="str">
+      <c r="B41" s="20" t="str">
         <f>IF(ISNA(MATCH(A41,RATE_DATE,0)),"",IF(INDEX(NF_RATE_MEDIAN,MATCH(A41,RATE_DATE,0))="","",INDEX(NF_RATE_MEDIAN,MATCH(A41,RATE_DATE,0))))</f>
         <v/>
       </c>
@@ -4524,7 +4523,7 @@
         <f>DATE(2018,7,1)</f>
         <v>43282</v>
       </c>
-      <c r="B42" s="21">
+      <c r="B42" s="20">
         <f>IF(ISNA(MATCH(A42,RATE_DATE,0)),"",IF(INDEX(NF_RATE_MEDIAN,MATCH(A42,RATE_DATE,0))="","",INDEX(NF_RATE_MEDIAN,MATCH(A42,RATE_DATE,0))))</f>
         <v>270.66</v>
       </c>
@@ -4538,7 +4537,7 @@
         <f>DATE(2019,1,1)</f>
         <v>43466</v>
       </c>
-      <c r="B43" s="21">
+      <c r="B43" s="20">
         <f>IF(ISNA(MATCH(A43,RATE_DATE,0)),"",IF(INDEX(NF_RATE_MEDIAN,MATCH(A43,RATE_DATE,0))="","",INDEX(NF_RATE_MEDIAN,MATCH(A43,RATE_DATE,0))))</f>
         <v>270.15</v>
       </c>
@@ -4552,7 +4551,7 @@
         <f>DATE(2019,7,1)</f>
         <v>43647</v>
       </c>
-      <c r="B44" s="21" t="str">
+      <c r="B44" s="20" t="str">
         <f>IF(ISNA(MATCH(A44,RATE_DATE,0)),"",IF(INDEX(NF_RATE_MEDIAN,MATCH(A44,RATE_DATE,0))="","",INDEX(NF_RATE_MEDIAN,MATCH(A44,RATE_DATE,0))))</f>
         <v/>
       </c>
@@ -4566,7 +4565,7 @@
         <f>DATE(2020,1,1)</f>
         <v>43831</v>
       </c>
-      <c r="B45" s="21" t="str">
+      <c r="B45" s="20" t="str">
         <f>IF(ISNA(MATCH(A45,RATE_DATE,0)),"",IF(INDEX(NF_RATE_MEDIAN,MATCH(A45,RATE_DATE,0))="","",INDEX(NF_RATE_MEDIAN,MATCH(A45,RATE_DATE,0))))</f>
         <v/>
       </c>
@@ -4580,7 +4579,7 @@
         <f>DATE(2020,7,1)</f>
         <v>44013</v>
       </c>
-      <c r="B46" s="21">
+      <c r="B46" s="20">
         <f>IF(ISNA(MATCH(A46,RATE_DATE,0)),"",IF(INDEX(NF_RATE_MEDIAN,MATCH(A46,RATE_DATE,0))="","",INDEX(NF_RATE_MEDIAN,MATCH(A46,RATE_DATE,0))))</f>
         <v>282.98</v>
       </c>
@@ -4594,7 +4593,7 @@
         <f>DATE(2021,1,1)</f>
         <v>44197</v>
       </c>
-      <c r="B47" s="21" t="str">
+      <c r="B47" s="20" t="str">
         <f>IF(ISNA(MATCH(A47,RATE_DATE,0)),"",IF(INDEX(NF_RATE_MEDIAN,MATCH(A47,RATE_DATE,0))="","",INDEX(NF_RATE_MEDIAN,MATCH(A47,RATE_DATE,0))))</f>
         <v/>
       </c>
@@ -4608,7 +4607,7 @@
         <f>DATE(2021,7,1)</f>
         <v>44378</v>
       </c>
-      <c r="B48" s="21">
+      <c r="B48" s="20">
         <f>IF(ISNA(MATCH(A48,RATE_DATE,0)),"",IF(INDEX(NF_RATE_MEDIAN,MATCH(A48,RATE_DATE,0))="","",INDEX(NF_RATE_MEDIAN,MATCH(A48,RATE_DATE,0))))</f>
         <v>334.75</v>
       </c>
@@ -4622,7 +4621,7 @@
         <f>DATE(2022,1,1)</f>
         <v>44562</v>
       </c>
-      <c r="B49" s="21">
+      <c r="B49" s="20">
         <f>IF(ISNA(MATCH(A49,RATE_DATE,0)),"",IF(INDEX(NF_RATE_MEDIAN,MATCH(A49,RATE_DATE,0))="","",INDEX(NF_RATE_MEDIAN,MATCH(A49,RATE_DATE,0))))</f>
         <v>332.59</v>
       </c>
@@ -4636,7 +4635,7 @@
         <f>DATE(2022,7,1)</f>
         <v>44743</v>
       </c>
-      <c r="B50" s="21" t="str">
+      <c r="B50" s="20" t="str">
         <f>IF(ISNA(MATCH(A50,RATE_DATE,0)),"",IF(INDEX(NF_RATE_MEDIAN,MATCH(A50,RATE_DATE,0))="","",INDEX(NF_RATE_MEDIAN,MATCH(A50,RATE_DATE,0))))</f>
         <v/>
       </c>
@@ -4650,7 +4649,7 @@
         <f>DATE(2023,1,1)</f>
         <v>44927</v>
       </c>
-      <c r="B51" s="21">
+      <c r="B51" s="20">
         <f>IF(ISNA(MATCH(A51,RATE_DATE,0)),"",IF(INDEX(NF_RATE_MEDIAN,MATCH(A51,RATE_DATE,0))="","",INDEX(NF_RATE_MEDIAN,MATCH(A51,RATE_DATE,0))))</f>
         <v>355.11</v>
       </c>
@@ -4664,7 +4663,7 @@
         <f>DATE(2023,7,1)</f>
         <v>45108</v>
       </c>
-      <c r="B52" s="21">
+      <c r="B52" s="20">
         <f>IF(ISNA(MATCH(A52,RATE_DATE,0)),"",IF(INDEX(NF_RATE_MEDIAN,MATCH(A52,RATE_DATE,0))="","",INDEX(NF_RATE_MEDIAN,MATCH(A52,RATE_DATE,0))))</f>
         <v>371.99</v>
       </c>
@@ -4678,7 +4677,7 @@
         <f>DATE(2024,1,1)</f>
         <v>45292</v>
       </c>
-      <c r="B53" s="21">
+      <c r="B53" s="20">
         <f>IF(ISNA(MATCH(A53,RATE_DATE,0)),"",IF(INDEX(NF_RATE_MEDIAN,MATCH(A53,RATE_DATE,0))="","",INDEX(NF_RATE_MEDIAN,MATCH(A53,RATE_DATE,0))))</f>
         <v>481.83</v>
       </c>
@@ -4692,7 +4691,7 @@
         <f>DATE(2024,7,1)</f>
         <v>45474</v>
       </c>
-      <c r="B54" s="21">
+      <c r="B54" s="20">
         <f>IF(ISNA(MATCH(A54,RATE_DATE,0)),"",IF(INDEX(NF_RATE_MEDIAN,MATCH(A54,RATE_DATE,0))="","",INDEX(NF_RATE_MEDIAN,MATCH(A54,RATE_DATE,0))))</f>
         <v>482.2</v>
       </c>
@@ -4706,7 +4705,7 @@
         <f>DATE(2025,1,1)</f>
         <v>45658</v>
       </c>
-      <c r="B55" s="21">
+      <c r="B55" s="20">
         <f>IF(ISNA(MATCH(A55,RATE_DATE,0)),"",IF(INDEX(NF_RATE_MEDIAN,MATCH(A55,RATE_DATE,0))="","",INDEX(NF_RATE_MEDIAN,MATCH(A55,RATE_DATE,0))))</f>
         <v>509.69</v>
       </c>
@@ -4720,7 +4719,7 @@
         <f>DATE(2025,7,1)</f>
         <v>45839</v>
       </c>
-      <c r="B56" s="21">
+      <c r="B56" s="20">
         <f>IF(ISNA(MATCH(A56,RATE_DATE,0)),"",IF(INDEX(NF_RATE_MEDIAN,MATCH(A56,RATE_DATE,0))="","",INDEX(NF_RATE_MEDIAN,MATCH(A56,RATE_DATE,0))))</f>
         <v>506.65</v>
       </c>
@@ -4734,7 +4733,7 @@
         <f>DATE(2026,1,1)</f>
         <v>46023</v>
       </c>
-      <c r="B57" s="21">
+      <c r="B57" s="20">
         <f>IF(ISNA(MATCH(A57,RATE_DATE,0)),"",IF(INDEX(NF_RATE_MEDIAN,MATCH(A57,RATE_DATE,0))="","",INDEX(NF_RATE_MEDIAN,MATCH(A57,RATE_DATE,0))))</f>
         <v>495.25</v>
       </c>
@@ -4777,15 +4776,15 @@
         <f>INDEX(COST_FY,1)</f>
         <v>2011</v>
       </c>
-      <c r="B61" s="25">
+      <c r="B61" s="22">
         <f>DATE(INDEX(COST_FY,1),7,1)</f>
         <v>40725</v>
       </c>
-      <c r="C61" s="21">
+      <c r="C61" s="20">
         <f>INDEX(NF_COST_MCD_HEAVY,1)</f>
         <v>287.76</v>
       </c>
-      <c r="D61" s="21">
+      <c r="D61" s="20">
         <f>INDEX(NF_COST_ALL,1)</f>
         <v>295.13</v>
       </c>
@@ -4795,15 +4794,15 @@
         <f>INDEX(COST_FY,2)</f>
         <v>2012</v>
       </c>
-      <c r="B62" s="25">
+      <c r="B62" s="22">
         <f>DATE(INDEX(COST_FY,2),7,1)</f>
         <v>41091</v>
       </c>
-      <c r="C62" s="21">
+      <c r="C62" s="20">
         <f>INDEX(NF_COST_MCD_HEAVY,2)</f>
         <v>311.89</v>
       </c>
-      <c r="D62" s="21">
+      <c r="D62" s="20">
         <f>INDEX(NF_COST_ALL,2)</f>
         <v>314.68</v>
       </c>
@@ -4813,15 +4812,15 @@
         <f>INDEX(COST_FY,3)</f>
         <v>2013</v>
       </c>
-      <c r="B63" s="25">
+      <c r="B63" s="22">
         <f>DATE(INDEX(COST_FY,3),7,1)</f>
         <v>41456</v>
       </c>
-      <c r="C63" s="21">
+      <c r="C63" s="20">
         <f>INDEX(NF_COST_MCD_HEAVY,3)</f>
         <v>322.2</v>
       </c>
-      <c r="D63" s="21">
+      <c r="D63" s="20">
         <f>INDEX(NF_COST_ALL,3)</f>
         <v>342.42</v>
       </c>
@@ -4831,15 +4830,15 @@
         <f>INDEX(COST_FY,4)</f>
         <v>2014</v>
       </c>
-      <c r="B64" s="25">
+      <c r="B64" s="22">
         <f>DATE(INDEX(COST_FY,4),7,1)</f>
         <v>41821</v>
       </c>
-      <c r="C64" s="21">
+      <c r="C64" s="20">
         <f>INDEX(NF_COST_MCD_HEAVY,4)</f>
         <v>322.2</v>
       </c>
-      <c r="D64" s="21">
+      <c r="D64" s="20">
         <f>INDEX(NF_COST_ALL,4)</f>
         <v>344.18</v>
       </c>
@@ -4849,15 +4848,15 @@
         <f>INDEX(COST_FY,5)</f>
         <v>2015</v>
       </c>
-      <c r="B65" s="25">
+      <c r="B65" s="22">
         <f>DATE(INDEX(COST_FY,5),7,1)</f>
         <v>42186</v>
       </c>
-      <c r="C65" s="21">
+      <c r="C65" s="20">
         <f>INDEX(NF_COST_MCD_HEAVY,5)</f>
         <v>322.11</v>
       </c>
-      <c r="D65" s="21">
+      <c r="D65" s="20">
         <f>INDEX(NF_COST_ALL,5)</f>
         <v>340.9</v>
       </c>
@@ -4867,15 +4866,15 @@
         <f>INDEX(COST_FY,6)</f>
         <v>2016</v>
       </c>
-      <c r="B66" s="25">
+      <c r="B66" s="22">
         <f>DATE(INDEX(COST_FY,6),7,1)</f>
         <v>42552</v>
       </c>
-      <c r="C66" s="21">
+      <c r="C66" s="20">
         <f>INDEX(NF_COST_MCD_HEAVY,6)</f>
         <v>344.38</v>
       </c>
-      <c r="D66" s="21">
+      <c r="D66" s="20">
         <f>INDEX(NF_COST_ALL,6)</f>
         <v>358.8</v>
       </c>
@@ -4885,15 +4884,15 @@
         <f>INDEX(COST_FY,7)</f>
         <v>2017</v>
       </c>
-      <c r="B67" s="25">
+      <c r="B67" s="22">
         <f>DATE(INDEX(COST_FY,7),7,1)</f>
         <v>42917</v>
       </c>
-      <c r="C67" s="21">
+      <c r="C67" s="20">
         <f>INDEX(NF_COST_MCD_HEAVY,7)</f>
         <v>356.1</v>
       </c>
-      <c r="D67" s="21">
+      <c r="D67" s="20">
         <f>INDEX(NF_COST_ALL,7)</f>
         <v>376.01</v>
       </c>
@@ -4903,15 +4902,15 @@
         <f>INDEX(COST_FY,8)</f>
         <v>2018</v>
       </c>
-      <c r="B68" s="25">
+      <c r="B68" s="22">
         <f>DATE(INDEX(COST_FY,8),7,1)</f>
         <v>43282</v>
       </c>
-      <c r="C68" s="21">
+      <c r="C68" s="20">
         <f>INDEX(NF_COST_MCD_HEAVY,8)</f>
         <v>365.93</v>
       </c>
-      <c r="D68" s="21">
+      <c r="D68" s="20">
         <f>INDEX(NF_COST_ALL,8)</f>
         <v>380.99</v>
       </c>
@@ -4921,15 +4920,15 @@
         <f>INDEX(COST_FY,9)</f>
         <v>2019</v>
       </c>
-      <c r="B69" s="25">
+      <c r="B69" s="22">
         <f>DATE(INDEX(COST_FY,9),7,1)</f>
         <v>43647</v>
       </c>
-      <c r="C69" s="21">
+      <c r="C69" s="20">
         <f>INDEX(NF_COST_MCD_HEAVY,9)</f>
         <v>373.25</v>
       </c>
-      <c r="D69" s="21">
+      <c r="D69" s="20">
         <f>INDEX(NF_COST_ALL,9)</f>
         <v>379.87</v>
       </c>
@@ -4939,15 +4938,15 @@
         <f>INDEX(COST_FY,10)</f>
         <v>2020</v>
       </c>
-      <c r="B70" s="25">
+      <c r="B70" s="22">
         <f>DATE(INDEX(COST_FY,10),7,1)</f>
         <v>44013</v>
       </c>
-      <c r="C70" s="21">
+      <c r="C70" s="20">
         <f>INDEX(NF_COST_MCD_HEAVY,10)</f>
         <v>398.33</v>
       </c>
-      <c r="D70" s="21">
+      <c r="D70" s="20">
         <f>INDEX(NF_COST_ALL,10)</f>
         <v>428.4</v>
       </c>
@@ -4957,15 +4956,15 @@
         <f>INDEX(COST_FY,11)</f>
         <v>2021</v>
       </c>
-      <c r="B71" s="25">
+      <c r="B71" s="22">
         <f>DATE(INDEX(COST_FY,11),7,1)</f>
         <v>44378</v>
       </c>
-      <c r="C71" s="21">
+      <c r="C71" s="20">
         <f>INDEX(NF_COST_MCD_HEAVY,11)</f>
         <v>423.44</v>
       </c>
-      <c r="D71" s="21">
+      <c r="D71" s="20">
         <f>INDEX(NF_COST_ALL,11)</f>
         <v>450.4</v>
       </c>
@@ -4975,15 +4974,15 @@
         <f>INDEX(COST_FY,12)</f>
         <v>2022</v>
       </c>
-      <c r="B72" s="25">
+      <c r="B72" s="22">
         <f>DATE(INDEX(COST_FY,12),7,1)</f>
         <v>44743</v>
       </c>
-      <c r="C72" s="21">
+      <c r="C72" s="20">
         <f>INDEX(NF_COST_MCD_HEAVY,12)</f>
         <v>435.63</v>
       </c>
-      <c r="D72" s="21">
+      <c r="D72" s="20">
         <f>INDEX(NF_COST_ALL,12)</f>
         <v>459.47</v>
       </c>
@@ -4993,15 +4992,15 @@
         <f>INDEX(COST_FY,13)</f>
         <v>2023</v>
       </c>
-      <c r="B73" s="25">
+      <c r="B73" s="22">
         <f>DATE(INDEX(COST_FY,13),7,1)</f>
         <v>45108</v>
       </c>
-      <c r="C73" s="21">
+      <c r="C73" s="20">
         <f>INDEX(NF_COST_MCD_HEAVY,13)</f>
         <v>461.78</v>
       </c>
-      <c r="D73" s="21">
+      <c r="D73" s="20">
         <f>INDEX(NF_COST_ALL,13)</f>
         <v>519.16</v>
       </c>
@@ -5201,10 +5200,10 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -5248,7 +5247,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="27">
+      <c r="A4" s="24">
         <f>1</f>
         <v>1</v>
       </c>
@@ -5257,11 +5256,11 @@
           <t>DAYS_PER_PT(2023)</t>
         </is>
       </c>
-      <c r="C4" s="18">
+      <c r="C4" s="25">
         <f>INDEX(DAYS_PER_PT,MATCH(2023,YEAR,0))</f>
         <v>23.018559556786702</v>
       </c>
-      <c r="D4" s="18">
+      <c r="D4" s="25">
         <f>23.02</f>
         <v>23.02</v>
       </c>
@@ -5275,7 +5274,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="27">
+      <c r="A5" s="24">
         <f>2</f>
         <v>2</v>
       </c>
@@ -5284,11 +5283,11 @@
           <t>DAYS_PER_PT(2024)</t>
         </is>
       </c>
-      <c r="C5" s="18">
+      <c r="C5" s="25">
         <f>INDEX(DAYS_PER_PT,MATCH(2024,YEAR,0))</f>
         <v>19.492795389048993</v>
       </c>
-      <c r="D5" s="18">
+      <c r="D5" s="25">
         <f>19.49</f>
         <v>19.49</v>
       </c>
@@ -5302,7 +5301,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="27">
+      <c r="A6" s="24">
         <f>3</f>
         <v>3</v>
       </c>
@@ -5329,7 +5328,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="27">
+      <c r="A7" s="24">
         <f>4</f>
         <v>4</v>
       </c>
@@ -5356,7 +5355,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="27">
+      <c r="A8" s="24">
         <f>5</f>
         <v>5</v>
       </c>
@@ -5383,7 +5382,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="27">
+      <c r="A9" s="24">
         <f>6</f>
         <v>6</v>
       </c>
@@ -5410,7 +5409,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="27">
+      <c r="A10" s="24">
         <f>7</f>
         <v>7</v>
       </c>
@@ -5437,7 +5436,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="27">
+      <c r="A11" s="24">
         <f>8</f>
         <v>8</v>
       </c>
@@ -5446,11 +5445,11 @@
           <t>GAP_PER_PT(2017)</t>
         </is>
       </c>
-      <c r="C11" s="18">
+      <c r="C11" s="25">
         <f>INDEX(GAP_PER_PT,MATCH(2017,YEAR,0))</f>
         <v>-4.064651689025375</v>
       </c>
-      <c r="D11" s="18">
+      <c r="D11" s="25">
         <f>-4.06</f>
         <v>-4.06</v>
       </c>
@@ -5464,7 +5463,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="27">
+      <c r="A12" s="24">
         <f>9</f>
         <v>9</v>
       </c>
@@ -5473,11 +5472,11 @@
           <t>GAP_PER_PT(2024)</t>
         </is>
       </c>
-      <c r="C12" s="18">
+      <c r="C12" s="25">
         <f>INDEX(GAP_PER_PT,MATCH(2024,YEAR,0))</f>
         <v>5.492795389048993</v>
       </c>
-      <c r="D12" s="18">
+      <c r="D12" s="25">
         <f>5.49</f>
         <v>5.49</v>
       </c>
@@ -5491,7 +5490,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="27">
+      <c r="A13" s="24">
         <f>10</f>
         <v>10</v>
       </c>
@@ -5500,11 +5499,11 @@
           <t>WL_RATE_AVG(2023)</t>
         </is>
       </c>
-      <c r="C13" s="22">
+      <c r="C13" s="26">
         <f>INDEX(WL_RATE_AVG,1)</f>
         <v>293.245</v>
       </c>
-      <c r="D13" s="22">
+      <c r="D13" s="26">
         <f>293.245</f>
         <v>293.245</v>
       </c>
@@ -5518,7 +5517,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="27">
+      <c r="A14" s="24">
         <f>11</f>
         <v>11</v>
       </c>
@@ -5527,11 +5526,11 @@
           <t>WL_RATE_AVG(2024)</t>
         </is>
       </c>
-      <c r="C14" s="22">
+      <c r="C14" s="26">
         <f>INDEX(WL_RATE_AVG,2)</f>
         <v>460.28</v>
       </c>
-      <c r="D14" s="22">
+      <c r="D14" s="26">
         <f>460.28</f>
         <v>460.28</v>
       </c>
@@ -5545,7 +5544,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="27">
+      <c r="A15" s="24">
         <f>12</f>
         <v>12</v>
       </c>
@@ -5554,11 +5553,11 @@
           <t>NET_COST_LO(2024)</t>
         </is>
       </c>
-      <c r="C15" s="21">
+      <c r="C15" s="20">
         <f>INDEX(NET_COST_LO,2)</f>
         <v>89.72000000000003</v>
       </c>
-      <c r="D15" s="21">
+      <c r="D15" s="20">
         <f>89.72</f>
         <v>89.72</v>
       </c>
@@ -5572,7 +5571,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="27">
+      <c r="A16" s="24">
         <f>13</f>
         <v>13</v>
       </c>
@@ -5581,11 +5580,11 @@
           <t>NET_COST_HI(2024)</t>
         </is>
       </c>
-      <c r="C16" s="21">
+      <c r="C16" s="20">
         <f>INDEX(NET_COST_HI,2)</f>
         <v>1009.72</v>
       </c>
-      <c r="D16" s="21">
+      <c r="D16" s="20">
         <f>1009.72</f>
         <v>1009.72</v>
       </c>
@@ -5599,7 +5598,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="27">
+      <c r="A17" s="24">
         <f>14</f>
         <v>14</v>
       </c>
@@ -5608,11 +5607,11 @@
           <t>EXCESS_COST_LO(2024) (about)</t>
         </is>
       </c>
-      <c r="C17" s="23">
+      <c r="C17" s="21">
         <f>INDEX(EXCESS_COST_LO,2)</f>
         <v>1539056.8800000004</v>
       </c>
-      <c r="D17" s="23">
+      <c r="D17" s="21">
         <f>1539057</f>
         <v>1539057</v>
       </c>
@@ -5626,7 +5625,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="27">
+      <c r="A18" s="24">
         <f>15</f>
         <v>15</v>
       </c>
@@ -5635,11 +5634,11 @@
           <t>EXCESS_COST_HI(2024) (about)</t>
         </is>
       </c>
-      <c r="C18" s="23">
+      <c r="C18" s="21">
         <f>INDEX(EXCESS_COST_HI,2)</f>
         <v>17320736.88</v>
       </c>
-      <c r="D18" s="23">
+      <c r="D18" s="21">
         <f>17320737</f>
         <v>17320737</v>
       </c>
@@ -5653,7 +5652,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="27">
+      <c r="A19" s="24">
         <f>16</f>
         <v>16</v>
       </c>
@@ -5662,11 +5661,11 @@
           <t>NET_COST_LO_NOW</t>
         </is>
       </c>
-      <c r="C19" s="21">
+      <c r="C19" s="20">
         <f>NET_COST_LO_NOW</f>
         <v>63.24000000000001</v>
       </c>
-      <c r="D19" s="21">
+      <c r="D19" s="20">
         <f>63.24</f>
         <v>63.24</v>
       </c>
@@ -5680,7 +5679,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="27">
+      <c r="A20" s="24">
         <f>17</f>
         <v>17</v>
       </c>
@@ -5689,11 +5688,11 @@
           <t>NET_COST_HI_NOW</t>
         </is>
       </c>
-      <c r="C20" s="21">
+      <c r="C20" s="20">
         <f>NET_COST_HI_NOW</f>
         <v>983.24</v>
       </c>
-      <c r="D20" s="21">
+      <c r="D20" s="20">
         <f>983.24</f>
         <v>983.24</v>
       </c>
@@ -5707,7 +5706,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="27">
+      <c r="A21" s="24">
         <f>18</f>
         <v>18</v>
       </c>
@@ -5716,11 +5715,11 @@
           <t>WL_DAYS_CHANGE_2024</t>
         </is>
       </c>
-      <c r="C21" s="19">
+      <c r="C21" s="18">
         <f>WL_DAYS_CHANGE_2024</f>
         <v>-0.26741037582584204</v>
       </c>
-      <c r="D21" s="19">
+      <c r="D21" s="18">
         <f>-0.267</f>
         <v>-0.267</v>
       </c>
@@ -5734,7 +5733,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="27">
+      <c r="A22" s="24">
         <f>19</f>
         <v>19</v>
       </c>
@@ -5743,11 +5742,11 @@
           <t>T1_DROP_2021 (points)</t>
         </is>
       </c>
-      <c r="C22" s="18">
+      <c r="C22" s="25">
         <f>T1_DROP_2021*100</f>
         <v>-1.917989417989416</v>
       </c>
-      <c r="D22" s="18">
+      <c r="D22" s="25">
         <f>-1.92</f>
         <v>-1.92</v>
       </c>
@@ -5761,7 +5760,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="27">
+      <c r="A23" s="24">
         <f>20</f>
         <v>20</v>
       </c>
@@ -5770,11 +5769,11 @@
           <t>T1_DROP_2024 (points)</t>
         </is>
       </c>
-      <c r="C23" s="18">
+      <c r="C23" s="25">
         <f>T1_DROP_2024*100</f>
         <v>-11.121871500771721</v>
       </c>
-      <c r="D23" s="18">
+      <c r="D23" s="25">
         <f>-11.12</f>
         <v>-11.12</v>
       </c>
@@ -5788,7 +5787,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="27">
+      <c r="A24" s="24">
         <f>21</f>
         <v>21</v>
       </c>
@@ -5797,11 +5796,11 @@
           <t>T2_SLOPE (about)</t>
         </is>
       </c>
-      <c r="C24" s="18">
+      <c r="C24" s="25">
         <f>T2_SLOPE</f>
         <v>1.8814212714379457</v>
       </c>
-      <c r="D24" s="18">
+      <c r="D24" s="25">
         <f>1.88</f>
         <v>1.88</v>
       </c>
@@ -5815,7 +5814,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="27">
+      <c r="A25" s="24">
         <f>22</f>
         <v>22</v>
       </c>
@@ -5842,7 +5841,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="27">
+      <c r="A26" s="24">
         <f>23</f>
         <v>23</v>
       </c>
@@ -5869,7 +5868,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="27">
+      <c r="A27" s="24">
         <f>24</f>
         <v>24</v>
       </c>
@@ -5896,7 +5895,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="27">
+      <c r="A28" s="24">
         <f>25</f>
         <v>25</v>
       </c>
@@ -5923,7 +5922,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="27">
+      <c r="A29" s="24">
         <f>26</f>
         <v>26</v>
       </c>
@@ -5950,7 +5949,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="27">
+      <c r="A30" s="24">
         <f>27</f>
         <v>27</v>
       </c>
@@ -5977,7 +5976,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="27">
+      <c r="A31" s="24">
         <f>28</f>
         <v>28</v>
       </c>
@@ -6004,7 +6003,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="27">
+      <c r="A32" s="24">
         <f>29</f>
         <v>29</v>
       </c>
@@ -6013,11 +6012,11 @@
           <t>KFF_COST_DAY x 0.15</t>
         </is>
       </c>
-      <c r="C32" s="21">
+      <c r="C32" s="20">
         <f>KFF_COST_DAY*0.15</f>
         <v>549.6</v>
       </c>
-      <c r="D32" s="21">
+      <c r="D32" s="20">
         <f>549.6</f>
         <v>549.6</v>
       </c>
@@ -6031,7 +6030,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="27">
+      <c r="A33" s="24">
         <f>30</f>
         <v>30</v>
       </c>
@@ -6040,11 +6039,11 @@
           <t>KFF_COST_DAY x 0.40</t>
         </is>
       </c>
-      <c r="C33" s="21">
+      <c r="C33" s="20">
         <f>KFF_COST_DAY*0.4</f>
         <v>1465.6000000000001</v>
       </c>
-      <c r="D33" s="21">
+      <c r="D33" s="20">
         <f>1465.6</f>
         <v>1465.6</v>
       </c>
@@ -6058,7 +6057,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="27">
+      <c r="A34" s="24">
         <f>31</f>
         <v>31</v>
       </c>
@@ -6067,11 +6066,11 @@
           <t>KFF_COST_DAY x 0.15 within rounding (to $10) of AVOID_COST_LO</t>
         </is>
       </c>
-      <c r="C34" s="21">
+      <c r="C34" s="20">
         <f>KFF_COST_DAY*0.15</f>
         <v>549.6</v>
       </c>
-      <c r="D34" s="21">
+      <c r="D34" s="20">
         <f>AVOID_COST_LO</f>
         <v>550</v>
       </c>
@@ -6085,7 +6084,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="27">
+      <c r="A35" s="24">
         <f>32</f>
         <v>32</v>
       </c>
@@ -6094,11 +6093,11 @@
           <t>KFF_COST_DAY x 0.40 within rounding (to $10) of AVOID_COST_HI</t>
         </is>
       </c>
-      <c r="C35" s="21">
+      <c r="C35" s="20">
         <f>KFF_COST_DAY*0.4</f>
         <v>1465.6000000000001</v>
       </c>
-      <c r="D35" s="21">
+      <c r="D35" s="20">
         <f>AVOID_COST_HI</f>
         <v>1470</v>
       </c>

</xml_diff>

<commit_message>
Compute the paper's rate rises, rate-cost gap and behavior and guardianship share in the model
A Paper figures block on the Conditions sheet: RATE_COST_GAP by fiscal
year with its smallest and largest value (19.45% to 28.96%),
RATE_RISE_2021 (18.3%), RATE_RISE_2024 (29.5%) and BEH_GUARD_SHARE_2024
(34.7%). Spec definitions, five anchors (50 in all) and the build record
updated. Model rebuilt: ALL PASS, 234 outputs with 0 mismatches.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/capabilities/economic-research/model.xlsx
+++ b/capabilities/economic-research/model.xlsx
@@ -112,6 +112,12 @@
     <definedName name="COND_A_GAP">'Conditions'!$E$7:$E$8</definedName>
     <definedName name="RATE_GROWTH_2024_2026">'Conditions'!$B$10</definedName>
     <definedName name="STAY_SHORTFALL">'Conditions'!$B$11</definedName>
+    <definedName name="RATE_COST_GAP">'Conditions'!$D$19:$D$26</definedName>
+    <definedName name="RATE_COST_GAP_MIN">'Conditions'!$B$28</definedName>
+    <definedName name="RATE_COST_GAP_MAX">'Conditions'!$B$29</definedName>
+    <definedName name="RATE_RISE_2021">'Conditions'!$B$31</definedName>
+    <definedName name="RATE_RISE_2024">'Conditions'!$B$32</definedName>
+    <definedName name="BEH_GUARD_SHARE_2024">'Conditions'!$B$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2913,7 +2919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G79"/>
+  <dimension ref="A1:G84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="7" min="1" max="1"/>
@@ -4416,291 +4422,291 @@
         <v>PASS</v>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" s="29">
+        <f>46</f>
+        <v>46</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Anchor</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>RATE_RISE_2021</t>
+        </is>
+      </c>
+      <c r="D50" s="20">
+        <f>RATE_RISE_2021</f>
+        <v>0.1829457912219945</v>
+      </c>
+      <c r="E50" s="20">
+        <f>0.183</f>
+        <v>0.183</v>
+      </c>
+      <c r="F50">
+        <f>0.0005</f>
+        <v>0.0005</v>
+      </c>
+      <c r="G50" t="str">
+        <f>IF(AND(ISNUMBER(D50),ISNUMBER(E50)),IF(ABS(D50-E50)&lt;=F50,"PASS","FAIL"),"FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
     <row r="51">
-      <c r="A51" s="4" t="inlineStr">
-        <is>
-          <t>Invariants (must pass for any inputs; part of ALL CHECKS)</t>
-        </is>
+      <c r="A51" s="29">
+        <f>47</f>
+        <v>47</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Anchor</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>RATE_RISE_2024</t>
+        </is>
+      </c>
+      <c r="D51" s="20">
+        <f>RATE_RISE_2024</f>
+        <v>0.29527675475147164</v>
+      </c>
+      <c r="E51" s="20">
+        <f>0.295</f>
+        <v>0.295</v>
+      </c>
+      <c r="F51">
+        <f>0.0005</f>
+        <v>0.0005</v>
+      </c>
+      <c r="G51" t="str">
+        <f>IF(AND(ISNUMBER(D51),ISNUMBER(E51)),IF(ABS(D51-E51)&lt;=F51,"PASS","FAIL"),"FAIL")</f>
+        <v>PASS</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="5" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B52" s="5" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="C52" s="5" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="inlineStr">
-        <is>
-          <t>Computed</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="inlineStr">
-        <is>
-          <t>Expected</t>
-        </is>
-      </c>
-      <c r="F52" s="5" t="inlineStr">
-        <is>
-          <t>Tolerance</t>
-        </is>
-      </c>
-      <c r="G52" s="5" t="inlineStr">
-        <is>
-          <t>Result</t>
-        </is>
+      <c r="A52" s="29">
+        <f>48</f>
+        <v>48</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Anchor</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>RATE_COST_GAP_MIN</t>
+        </is>
+      </c>
+      <c r="D52" s="26">
+        <f>RATE_COST_GAP_MIN</f>
+        <v>0.19446068559301843</v>
+      </c>
+      <c r="E52" s="26">
+        <f>0.1945</f>
+        <v>0.1945</v>
+      </c>
+      <c r="F52">
+        <f>5e-05</f>
+        <v>5e-05</v>
+      </c>
+      <c r="G52" t="str">
+        <f>IF(AND(ISNUMBER(D52),ISNUMBER(E52)),IF(ABS(D52-E52)&lt;=F52,"PASS","FAIL"),"FAIL")</f>
+        <v>PASS</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="29">
+        <f>49</f>
+        <v>49</v>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Anchor</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>RATE_COST_GAP_MAX</t>
+        </is>
+      </c>
+      <c r="D53" s="26">
+        <f>RATE_COST_GAP_MAX</f>
+        <v>0.289584013255341</v>
+      </c>
+      <c r="E53" s="26">
+        <f>0.2896</f>
+        <v>0.2896</v>
+      </c>
+      <c r="F53">
+        <f>5e-05</f>
+        <v>5e-05</v>
+      </c>
+      <c r="G53" t="str">
+        <f>IF(AND(ISNUMBER(D53),ISNUMBER(E53)),IF(ABS(D53-E53)&lt;=F53,"PASS","FAIL"),"FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="29">
+        <f>50</f>
+        <v>50</v>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Anchor</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>BEH_GUARD_SHARE_2024</t>
+        </is>
+      </c>
+      <c r="D54" s="20">
+        <f>BEH_GUARD_SHARE_2024</f>
+        <v>0.3468208092485549</v>
+      </c>
+      <c r="E54" s="20">
+        <f>0.347</f>
+        <v>0.347</v>
+      </c>
+      <c r="F54">
+        <f>0.0005</f>
+        <v>0.0005</v>
+      </c>
+      <c r="G54" t="str">
+        <f>IF(AND(ISNUMBER(D54),ISNUMBER(E54)),IF(ABS(D54-E54)&lt;=F54,"PASS","FAIL"),"FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Invariants (must pass for any inputs; part of ALL CHECKS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Computed</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>Tolerance</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="29">
         <f>1</f>
         <v>1</v>
       </c>
-      <c r="B53" s="2" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>I1</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr">
         <is>
           <t>The seven SHARE_ values sum to 1, every year</t>
         </is>
       </c>
-      <c r="D53" t="b">
+      <c r="D58" t="b">
         <f>AND(ABS(INDEX(SHARE_NO_BED,1)+INDEX(SHARE_BEHAVIOR,1)+INDEX(SHARE_SPECIAL_CARE,1)+INDEX(SHARE_FINANCIAL,1)+INDEX(SHARE_GUARDIANSHIP,1)+INDEX(SHARE_PASARR,1)+INDEX(SHARE_OTHER,1)-1)&lt;=1e-06,ABS(INDEX(SHARE_NO_BED,2)+INDEX(SHARE_BEHAVIOR,2)+INDEX(SHARE_SPECIAL_CARE,2)+INDEX(SHARE_FINANCIAL,2)+INDEX(SHARE_GUARDIANSHIP,2)+INDEX(SHARE_PASARR,2)+INDEX(SHARE_OTHER,2)-1)&lt;=1e-06,ABS(INDEX(SHARE_NO_BED,3)+INDEX(SHARE_BEHAVIOR,3)+INDEX(SHARE_SPECIAL_CARE,3)+INDEX(SHARE_FINANCIAL,3)+INDEX(SHARE_GUARDIANSHIP,3)+INDEX(SHARE_PASARR,3)+INDEX(SHARE_OTHER,3)-1)&lt;=1e-06,ABS(INDEX(SHARE_NO_BED,4)+INDEX(SHARE_BEHAVIOR,4)+INDEX(SHARE_SPECIAL_CARE,4)+INDEX(SHARE_FINANCIAL,4)+INDEX(SHARE_GUARDIANSHIP,4)+INDEX(SHARE_PASARR,4)+INDEX(SHARE_OTHER,4)-1)&lt;=1e-06,ABS(INDEX(SHARE_NO_BED,5)+INDEX(SHARE_BEHAVIOR,5)+INDEX(SHARE_SPECIAL_CARE,5)+INDEX(SHARE_FINANCIAL,5)+INDEX(SHARE_GUARDIANSHIP,5)+INDEX(SHARE_PASARR,5)+INDEX(SHARE_OTHER,5)-1)&lt;=1e-06,ABS(INDEX(SHARE_NO_BED,6)+INDEX(SHARE_BEHAVIOR,6)+INDEX(SHARE_SPECIAL_CARE,6)+INDEX(SHARE_FINANCIAL,6)+INDEX(SHARE_GUARDIANSHIP,6)+INDEX(SHARE_PASARR,6)+INDEX(SHARE_OTHER,6)-1)&lt;=1e-06,ABS(INDEX(SHARE_NO_BED,7)+INDEX(SHARE_BEHAVIOR,7)+INDEX(SHARE_SPECIAL_CARE,7)+INDEX(SHARE_FINANCIAL,7)+INDEX(SHARE_GUARDIANSHIP,7)+INDEX(SHARE_PASARR,7)+INDEX(SHARE_OTHER,7)-1)&lt;=1e-06,ABS(INDEX(SHARE_NO_BED,8)+INDEX(SHARE_BEHAVIOR,8)+INDEX(SHARE_SPECIAL_CARE,8)+INDEX(SHARE_FINANCIAL,8)+INDEX(SHARE_GUARDIANSHIP,8)+INDEX(SHARE_PASARR,8)+INDEX(SHARE_OTHER,8)-1)&lt;=1e-06)</f>
         <v>1</v>
       </c>
-      <c r="E53" t="b">
+      <c r="E58" t="b">
         <f>TRUE</f>
         <v>1</v>
       </c>
-      <c r="F53" t="str">
+      <c r="F58" t="str">
         <f>"exact"</f>
         <v>exact</v>
       </c>
-      <c r="G53" t="str">
-        <f>IF(D53=E53,"PASS","FAIL")</f>
+      <c r="G58" t="str">
+        <f>IF(D58=E58,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="29">
+    <row r="59">
+      <c r="A59" s="29">
         <f>2</f>
         <v>2</v>
       </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="B59" s="2" t="inlineStr">
         <is>
           <t>I2</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
+      <c r="C59" s="2" t="inlineStr">
         <is>
           <t>WITHIN_DAYS + EXCESS_DAYS = WL_DAYS, every year</t>
         </is>
       </c>
-      <c r="D54" t="b">
+      <c r="D59" t="b">
         <f>AND(ABS(INDEX(WITHIN_DAYS,1)+INDEX(EXCESS_DAYS,1)-INDEX(WL_DAYS,1))&lt;=1e-06,ABS(INDEX(WITHIN_DAYS,2)+INDEX(EXCESS_DAYS,2)-INDEX(WL_DAYS,2))&lt;=1e-06,ABS(INDEX(WITHIN_DAYS,3)+INDEX(EXCESS_DAYS,3)-INDEX(WL_DAYS,3))&lt;=1e-06,ABS(INDEX(WITHIN_DAYS,4)+INDEX(EXCESS_DAYS,4)-INDEX(WL_DAYS,4))&lt;=1e-06,ABS(INDEX(WITHIN_DAYS,5)+INDEX(EXCESS_DAYS,5)-INDEX(WL_DAYS,5))&lt;=1e-06,ABS(INDEX(WITHIN_DAYS,6)+INDEX(EXCESS_DAYS,6)-INDEX(WL_DAYS,6))&lt;=1e-06,ABS(INDEX(WITHIN_DAYS,7)+INDEX(EXCESS_DAYS,7)-INDEX(WL_DAYS,7))&lt;=1e-06,ABS(INDEX(WITHIN_DAYS,8)+INDEX(EXCESS_DAYS,8)-INDEX(WL_DAYS,8))&lt;=1e-06)</f>
         <v>1</v>
       </c>
-      <c r="E54" t="b">
+      <c r="E59" t="b">
         <f>TRUE</f>
         <v>1</v>
       </c>
-      <c r="F54" t="str">
+      <c r="F59" t="str">
         <f>"exact"</f>
         <v>exact</v>
       </c>
-      <c r="G54" t="str">
-        <f>IF(D54=E54,"PASS","FAIL")</f>
+      <c r="G59" t="str">
+        <f>IF(D59=E59,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="29">
+    <row r="60">
+      <c r="A60" s="29">
         <f>3</f>
         <v>3</v>
       </c>
-      <c r="B55" s="2" t="inlineStr">
+      <c r="B60" s="2" t="inlineStr">
         <is>
           <t>I3</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr">
         <is>
           <t>EXCESS_DAYS = MAX(0, GAP_PER_PT x WL_PATIENTS), every year (covers 2019 and 2022)</t>
         </is>
       </c>
-      <c r="D55" t="b">
+      <c r="D60" t="b">
         <f>AND(ABS(INDEX(EXCESS_DAYS,1)-MAX(0,INDEX(GAP_PER_PT,1)*INDEX(WL_PATIENTS,1)))&lt;=1e-06,ABS(INDEX(EXCESS_DAYS,2)-MAX(0,INDEX(GAP_PER_PT,2)*INDEX(WL_PATIENTS,2)))&lt;=1e-06,ABS(INDEX(EXCESS_DAYS,3)-MAX(0,INDEX(GAP_PER_PT,3)*INDEX(WL_PATIENTS,3)))&lt;=1e-06,ABS(INDEX(EXCESS_DAYS,4)-MAX(0,INDEX(GAP_PER_PT,4)*INDEX(WL_PATIENTS,4)))&lt;=1e-06,ABS(INDEX(EXCESS_DAYS,5)-MAX(0,INDEX(GAP_PER_PT,5)*INDEX(WL_PATIENTS,5)))&lt;=1e-06,ABS(INDEX(EXCESS_DAYS,6)-MAX(0,INDEX(GAP_PER_PT,6)*INDEX(WL_PATIENTS,6)))&lt;=1e-06,ABS(INDEX(EXCESS_DAYS,7)-MAX(0,INDEX(GAP_PER_PT,7)*INDEX(WL_PATIENTS,7)))&lt;=1e-06,ABS(INDEX(EXCESS_DAYS,8)-MAX(0,INDEX(GAP_PER_PT,8)*INDEX(WL_PATIENTS,8)))&lt;=1e-06)</f>
-        <v>1</v>
-      </c>
-      <c r="E55" t="b">
-        <f>TRUE</f>
-        <v>1</v>
-      </c>
-      <c r="F55" t="str">
-        <f>"exact"</f>
-        <v>exact</v>
-      </c>
-      <c r="G55" t="str">
-        <f>IF(D55=E55,"PASS","FAIL")</f>
-        <v>PASS</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="29">
-        <f>4</f>
-        <v>4</v>
-      </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>I4</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>County CTY_DAYS sum to WL_DAYS, 2023 and 2024</t>
-        </is>
-      </c>
-      <c r="D56" t="b">
-        <f>AND(ABS(INDEX(CTY_DAYS,1,1)+INDEX(CTY_DAYS,2,1)+INDEX(CTY_DAYS,3,1)+INDEX(CTY_DAYS,4,1)-INDEX(WL_DAYS,MATCH(2023,YEAR,0)))&lt;=1e-06,ABS(INDEX(CTY_DAYS,1,2)+INDEX(CTY_DAYS,2,2)+INDEX(CTY_DAYS,3,2)+INDEX(CTY_DAYS,4,2)-INDEX(WL_DAYS,MATCH(2024,YEAR,0)))&lt;=1e-06)</f>
-        <v>1</v>
-      </c>
-      <c r="E56" t="b">
-        <f>TRUE</f>
-        <v>1</v>
-      </c>
-      <c r="F56" t="str">
-        <f>"exact"</f>
-        <v>exact</v>
-      </c>
-      <c r="G56" t="str">
-        <f>IF(D56=E56,"PASS","FAIL")</f>
-        <v>PASS</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="29">
-        <f>5</f>
-        <v>5</v>
-      </c>
-      <c r="B57" s="2" t="inlineStr">
-        <is>
-          <t>I5</t>
-        </is>
-      </c>
-      <c r="C57" s="2" t="inlineStr">
-        <is>
-          <t>County CTY_DAY_SHARE sum to 1, 2023 and 2024</t>
-        </is>
-      </c>
-      <c r="D57" t="b">
-        <f>AND(ABS(INDEX(CTY_DAY_SHARE,1,1)+INDEX(CTY_DAY_SHARE,2,1)+INDEX(CTY_DAY_SHARE,3,1)+INDEX(CTY_DAY_SHARE,4,1)-1)&lt;=1e-06,ABS(INDEX(CTY_DAY_SHARE,1,2)+INDEX(CTY_DAY_SHARE,2,2)+INDEX(CTY_DAY_SHARE,3,2)+INDEX(CTY_DAY_SHARE,4,2)-1)&lt;=1e-06)</f>
-        <v>1</v>
-      </c>
-      <c r="E57" t="b">
-        <f>TRUE</f>
-        <v>1</v>
-      </c>
-      <c r="F57" t="str">
-        <f>"exact"</f>
-        <v>exact</v>
-      </c>
-      <c r="G57" t="str">
-        <f>IF(D57=E57,"PASS","FAIL")</f>
-        <v>PASS</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="29">
-        <f>6</f>
-        <v>6</v>
-      </c>
-      <c r="B58" s="2" t="inlineStr">
-        <is>
-          <t>I6</t>
-        </is>
-      </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>T2_SLOPE = least-squares slope written out by hand, 2017 to 2023</t>
-        </is>
-      </c>
-      <c r="D58" s="24">
-        <f>((INDEX(YEAR,1)-AVERAGE(INDEX(YEAR,1):INDEX(YEAR,7)))*(INDEX(DAYS_PER_PT,1)-AVERAGE(INDEX(DAYS_PER_PT,1):INDEX(DAYS_PER_PT,7)))+(INDEX(YEAR,2)-AVERAGE(INDEX(YEAR,1):INDEX(YEAR,7)))*(INDEX(DAYS_PER_PT,2)-AVERAGE(INDEX(DAYS_PER_PT,1):INDEX(DAYS_PER_PT,7)))+(INDEX(YEAR,3)-AVERAGE(INDEX(YEAR,1):INDEX(YEAR,7)))*(INDEX(DAYS_PER_PT,3)-AVERAGE(INDEX(DAYS_PER_PT,1):INDEX(DAYS_PER_PT,7)))+(INDEX(YEAR,4)-AVERAGE(INDEX(YEAR,1):INDEX(YEAR,7)))*(INDEX(DAYS_PER_PT,4)-AVERAGE(INDEX(DAYS_PER_PT,1):INDEX(DAYS_PER_PT,7)))+(INDEX(YEAR,5)-AVERAGE(INDEX(YEAR,1):INDEX(YEAR,7)))*(INDEX(DAYS_PER_PT,5)-AVERAGE(INDEX(DAYS_PER_PT,1):INDEX(DAYS_PER_PT,7)))+(INDEX(YEAR,6)-AVERAGE(INDEX(YEAR,1):INDEX(YEAR,7)))*(INDEX(DAYS_PER_PT,6)-AVERAGE(INDEX(DAYS_PER_PT,1):INDEX(DAYS_PER_PT,7)))+(INDEX(YEAR,7)-AVERAGE(INDEX(YEAR,1):INDEX(YEAR,7)))*(INDEX(DAYS_PER_PT,7)-AVERAGE(INDEX(DAYS_PER_PT,1):INDEX(DAYS_PER_PT,7))))/((INDEX(YEAR,1)-AVERAGE(INDEX(YEAR,1):INDEX(YEAR,7)))^2+(INDEX(YEAR,2)-AVERAGE(INDEX(YEAR,1):INDEX(YEAR,7)))^2+(INDEX(YEAR,3)-AVERAGE(INDEX(YEAR,1):INDEX(YEAR,7)))^2+(INDEX(YEAR,4)-AVERAGE(INDEX(YEAR,1):INDEX(YEAR,7)))^2+(INDEX(YEAR,5)-AVERAGE(INDEX(YEAR,1):INDEX(YEAR,7)))^2+(INDEX(YEAR,6)-AVERAGE(INDEX(YEAR,1):INDEX(YEAR,7)))^2+(INDEX(YEAR,7)-AVERAGE(INDEX(YEAR,1):INDEX(YEAR,7)))^2)</f>
-        <v>1.8814212714379457</v>
-      </c>
-      <c r="E58" s="24">
-        <f>T2_SLOPE</f>
-        <v>1.8814212714379457</v>
-      </c>
-      <c r="F58">
-        <f>1e-06</f>
-        <v>1e-06</v>
-      </c>
-      <c r="G58" t="str">
-        <f>IF(AND(ISNUMBER(D58),ISNUMBER(E58)),IF(ABS(D58-E58)&lt;=F58,"PASS","FAIL"),"FAIL")</f>
-        <v>PASS</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="29">
-        <f>7</f>
-        <v>7</v>
-      </c>
-      <c r="B59" s="2" t="inlineStr">
-        <is>
-          <t>I7</t>
-        </is>
-      </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>T3_YEARS recomputed from the counts (no bed above each other reason)</t>
-        </is>
-      </c>
-      <c r="D59" s="3">
-        <f>IF(AND(INDEX(REASON_NO_BED,1)&gt;INDEX(REASON_BEHAVIOR,1),INDEX(REASON_NO_BED,1)&gt;INDEX(REASON_SPECIAL_CARE,1),INDEX(REASON_NO_BED,1)&gt;INDEX(REASON_FINANCIAL,1),INDEX(REASON_NO_BED,1)&gt;INDEX(REASON_GUARDIANSHIP,1),INDEX(REASON_NO_BED,1)&gt;INDEX(REASON_PASARR,1),INDEX(REASON_NO_BED,1)&gt;INDEX(REASON_OTHER,1)),1,0)+IF(AND(INDEX(REASON_NO_BED,2)&gt;INDEX(REASON_BEHAVIOR,2),INDEX(REASON_NO_BED,2)&gt;INDEX(REASON_SPECIAL_CARE,2),INDEX(REASON_NO_BED,2)&gt;INDEX(REASON_FINANCIAL,2),INDEX(REASON_NO_BED,2)&gt;INDEX(REASON_GUARDIANSHIP,2),INDEX(REASON_NO_BED,2)&gt;INDEX(REASON_PASARR,2),INDEX(REASON_NO_BED,2)&gt;INDEX(REASON_OTHER,2)),1,0)+IF(AND(INDEX(REASON_NO_BED,3)&gt;INDEX(REASON_BEHAVIOR,3),INDEX(REASON_NO_BED,3)&gt;INDEX(REASON_SPECIAL_CARE,3),INDEX(REASON_NO_BED,3)&gt;INDEX(REASON_FINANCIAL,3),INDEX(REASON_NO_BED,3)&gt;INDEX(REASON_GUARDIANSHIP,3),INDEX(REASON_NO_BED,3)&gt;INDEX(REASON_PASARR,3),INDEX(REASON_NO_BED,3)&gt;INDEX(REASON_OTHER,3)),1,0)+IF(AND(INDEX(REASON_NO_BED,4)&gt;INDEX(REASON_BEHAVIOR,4),INDEX(REASON_NO_BED,4)&gt;INDEX(REASON_SPECIAL_CARE,4),INDEX(REASON_NO_BED,4)&gt;INDEX(REASON_FINANCIAL,4),INDEX(REASON_NO_BED,4)&gt;INDEX(REASON_GUARDIANSHIP,4),INDEX(REASON_NO_BED,4)&gt;INDEX(REASON_PASARR,4),INDEX(REASON_NO_BED,4)&gt;INDEX(REASON_OTHER,4)),1,0)+IF(AND(INDEX(REASON_NO_BED,5)&gt;INDEX(REASON_BEHAVIOR,5),INDEX(REASON_NO_BED,5)&gt;INDEX(REASON_SPECIAL_CARE,5),INDEX(REASON_NO_BED,5)&gt;INDEX(REASON_FINANCIAL,5),INDEX(REASON_NO_BED,5)&gt;INDEX(REASON_GUARDIANSHIP,5),INDEX(REASON_NO_BED,5)&gt;INDEX(REASON_PASARR,5),INDEX(REASON_NO_BED,5)&gt;INDEX(REASON_OTHER,5)),1,0)+IF(AND(INDEX(REASON_NO_BED,6)&gt;INDEX(REASON_BEHAVIOR,6),INDEX(REASON_NO_BED,6)&gt;INDEX(REASON_SPECIAL_CARE,6),INDEX(REASON_NO_BED,6)&gt;INDEX(REASON_FINANCIAL,6),INDEX(REASON_NO_BED,6)&gt;INDEX(REASON_GUARDIANSHIP,6),INDEX(REASON_NO_BED,6)&gt;INDEX(REASON_PASARR,6),INDEX(REASON_NO_BED,6)&gt;INDEX(REASON_OTHER,6)),1,0)+IF(AND(INDEX(REASON_NO_BED,7)&gt;INDEX(REASON_BEHAVIOR,7),INDEX(REASON_NO_BED,7)&gt;INDEX(REASON_SPECIAL_CARE,7),INDEX(REASON_NO_BED,7)&gt;INDEX(REASON_FINANCIAL,7),INDEX(REASON_NO_BED,7)&gt;INDEX(REASON_GUARDIANSHIP,7),INDEX(REASON_NO_BED,7)&gt;INDEX(REASON_PASARR,7),INDEX(REASON_NO_BED,7)&gt;INDEX(REASON_OTHER,7)),1,0)+IF(AND(INDEX(REASON_NO_BED,8)&gt;INDEX(REASON_BEHAVIOR,8),INDEX(REASON_NO_BED,8)&gt;INDEX(REASON_SPECIAL_CARE,8),INDEX(REASON_NO_BED,8)&gt;INDEX(REASON_FINANCIAL,8),INDEX(REASON_NO_BED,8)&gt;INDEX(REASON_GUARDIANSHIP,8),INDEX(REASON_NO_BED,8)&gt;INDEX(REASON_PASARR,8),INDEX(REASON_NO_BED,8)&gt;INDEX(REASON_OTHER,8)),1,0)</f>
-        <v>5.0</v>
-      </c>
-      <c r="E59" s="3">
-        <f>T3_YEARS</f>
-        <v>5</v>
-      </c>
-      <c r="F59">
-        <f>0</f>
-        <v>0</v>
-      </c>
-      <c r="G59" t="str">
-        <f>IF(AND(ISNUMBER(D59),ISNUMBER(E59)),IF(ABS(D59-E59)&lt;=F59,"PASS","FAIL"),"FAIL")</f>
-        <v>PASS</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="29">
-        <f>8</f>
-        <v>8</v>
-      </c>
-      <c r="B60" s="2" t="inlineStr">
-        <is>
-          <t>I8</t>
-        </is>
-      </c>
-      <c r="C60" s="2" t="inlineStr">
-        <is>
-          <t>MEETS_BENCH is TRUE exactly when GAP_PER_PT &lt;= 0, every year</t>
-        </is>
-      </c>
-      <c r="D60" t="b">
-        <f>AND(INDEX(MEETS_BENCH,1)=(INDEX(GAP_PER_PT,1)&lt;=0),INDEX(MEETS_BENCH,2)=(INDEX(GAP_PER_PT,2)&lt;=0),INDEX(MEETS_BENCH,3)=(INDEX(GAP_PER_PT,3)&lt;=0),INDEX(MEETS_BENCH,4)=(INDEX(GAP_PER_PT,4)&lt;=0),INDEX(MEETS_BENCH,5)=(INDEX(GAP_PER_PT,5)&lt;=0),INDEX(MEETS_BENCH,6)=(INDEX(GAP_PER_PT,6)&lt;=0),INDEX(MEETS_BENCH,7)=(INDEX(GAP_PER_PT,7)&lt;=0),INDEX(MEETS_BENCH,8)=(INDEX(GAP_PER_PT,8)&lt;=0))</f>
         <v>1</v>
       </c>
       <c r="E60" t="b">
@@ -4718,134 +4724,186 @@
     </row>
     <row r="61">
       <c r="A61" s="29">
+        <f>4</f>
+        <v>4</v>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>I4</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>County CTY_DAYS sum to WL_DAYS, 2023 and 2024</t>
+        </is>
+      </c>
+      <c r="D61" t="b">
+        <f>AND(ABS(INDEX(CTY_DAYS,1,1)+INDEX(CTY_DAYS,2,1)+INDEX(CTY_DAYS,3,1)+INDEX(CTY_DAYS,4,1)-INDEX(WL_DAYS,MATCH(2023,YEAR,0)))&lt;=1e-06,ABS(INDEX(CTY_DAYS,1,2)+INDEX(CTY_DAYS,2,2)+INDEX(CTY_DAYS,3,2)+INDEX(CTY_DAYS,4,2)-INDEX(WL_DAYS,MATCH(2024,YEAR,0)))&lt;=1e-06)</f>
+        <v>1</v>
+      </c>
+      <c r="E61" t="b">
+        <f>TRUE</f>
+        <v>1</v>
+      </c>
+      <c r="F61" t="str">
+        <f>"exact"</f>
+        <v>exact</v>
+      </c>
+      <c r="G61" t="str">
+        <f>IF(D61=E61,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="29">
+        <f>5</f>
+        <v>5</v>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>I5</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>County CTY_DAY_SHARE sum to 1, 2023 and 2024</t>
+        </is>
+      </c>
+      <c r="D62" t="b">
+        <f>AND(ABS(INDEX(CTY_DAY_SHARE,1,1)+INDEX(CTY_DAY_SHARE,2,1)+INDEX(CTY_DAY_SHARE,3,1)+INDEX(CTY_DAY_SHARE,4,1)-1)&lt;=1e-06,ABS(INDEX(CTY_DAY_SHARE,1,2)+INDEX(CTY_DAY_SHARE,2,2)+INDEX(CTY_DAY_SHARE,3,2)+INDEX(CTY_DAY_SHARE,4,2)-1)&lt;=1e-06)</f>
+        <v>1</v>
+      </c>
+      <c r="E62" t="b">
+        <f>TRUE</f>
+        <v>1</v>
+      </c>
+      <c r="F62" t="str">
+        <f>"exact"</f>
+        <v>exact</v>
+      </c>
+      <c r="G62" t="str">
+        <f>IF(D62=E62,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="29">
+        <f>6</f>
+        <v>6</v>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>I6</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>T2_SLOPE = least-squares slope written out by hand, 2017 to 2023</t>
+        </is>
+      </c>
+      <c r="D63" s="24">
+        <f>((INDEX(YEAR,1)-AVERAGE(INDEX(YEAR,1):INDEX(YEAR,7)))*(INDEX(DAYS_PER_PT,1)-AVERAGE(INDEX(DAYS_PER_PT,1):INDEX(DAYS_PER_PT,7)))+(INDEX(YEAR,2)-AVERAGE(INDEX(YEAR,1):INDEX(YEAR,7)))*(INDEX(DAYS_PER_PT,2)-AVERAGE(INDEX(DAYS_PER_PT,1):INDEX(DAYS_PER_PT,7)))+(INDEX(YEAR,3)-AVERAGE(INDEX(YEAR,1):INDEX(YEAR,7)))*(INDEX(DAYS_PER_PT,3)-AVERAGE(INDEX(DAYS_PER_PT,1):INDEX(DAYS_PER_PT,7)))+(INDEX(YEAR,4)-AVERAGE(INDEX(YEAR,1):INDEX(YEAR,7)))*(INDEX(DAYS_PER_PT,4)-AVERAGE(INDEX(DAYS_PER_PT,1):INDEX(DAYS_PER_PT,7)))+(INDEX(YEAR,5)-AVERAGE(INDEX(YEAR,1):INDEX(YEAR,7)))*(INDEX(DAYS_PER_PT,5)-AVERAGE(INDEX(DAYS_PER_PT,1):INDEX(DAYS_PER_PT,7)))+(INDEX(YEAR,6)-AVERAGE(INDEX(YEAR,1):INDEX(YEAR,7)))*(INDEX(DAYS_PER_PT,6)-AVERAGE(INDEX(DAYS_PER_PT,1):INDEX(DAYS_PER_PT,7)))+(INDEX(YEAR,7)-AVERAGE(INDEX(YEAR,1):INDEX(YEAR,7)))*(INDEX(DAYS_PER_PT,7)-AVERAGE(INDEX(DAYS_PER_PT,1):INDEX(DAYS_PER_PT,7))))/((INDEX(YEAR,1)-AVERAGE(INDEX(YEAR,1):INDEX(YEAR,7)))^2+(INDEX(YEAR,2)-AVERAGE(INDEX(YEAR,1):INDEX(YEAR,7)))^2+(INDEX(YEAR,3)-AVERAGE(INDEX(YEAR,1):INDEX(YEAR,7)))^2+(INDEX(YEAR,4)-AVERAGE(INDEX(YEAR,1):INDEX(YEAR,7)))^2+(INDEX(YEAR,5)-AVERAGE(INDEX(YEAR,1):INDEX(YEAR,7)))^2+(INDEX(YEAR,6)-AVERAGE(INDEX(YEAR,1):INDEX(YEAR,7)))^2+(INDEX(YEAR,7)-AVERAGE(INDEX(YEAR,1):INDEX(YEAR,7)))^2)</f>
+        <v>1.8814212714379457</v>
+      </c>
+      <c r="E63" s="24">
+        <f>T2_SLOPE</f>
+        <v>1.8814212714379457</v>
+      </c>
+      <c r="F63">
+        <f>1e-06</f>
+        <v>1e-06</v>
+      </c>
+      <c r="G63" t="str">
+        <f>IF(AND(ISNUMBER(D63),ISNUMBER(E63)),IF(ABS(D63-E63)&lt;=F63,"PASS","FAIL"),"FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="29">
+        <f>7</f>
+        <v>7</v>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>I7</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>T3_YEARS recomputed from the counts (no bed above each other reason)</t>
+        </is>
+      </c>
+      <c r="D64" s="3">
+        <f>IF(AND(INDEX(REASON_NO_BED,1)&gt;INDEX(REASON_BEHAVIOR,1),INDEX(REASON_NO_BED,1)&gt;INDEX(REASON_SPECIAL_CARE,1),INDEX(REASON_NO_BED,1)&gt;INDEX(REASON_FINANCIAL,1),INDEX(REASON_NO_BED,1)&gt;INDEX(REASON_GUARDIANSHIP,1),INDEX(REASON_NO_BED,1)&gt;INDEX(REASON_PASARR,1),INDEX(REASON_NO_BED,1)&gt;INDEX(REASON_OTHER,1)),1,0)+IF(AND(INDEX(REASON_NO_BED,2)&gt;INDEX(REASON_BEHAVIOR,2),INDEX(REASON_NO_BED,2)&gt;INDEX(REASON_SPECIAL_CARE,2),INDEX(REASON_NO_BED,2)&gt;INDEX(REASON_FINANCIAL,2),INDEX(REASON_NO_BED,2)&gt;INDEX(REASON_GUARDIANSHIP,2),INDEX(REASON_NO_BED,2)&gt;INDEX(REASON_PASARR,2),INDEX(REASON_NO_BED,2)&gt;INDEX(REASON_OTHER,2)),1,0)+IF(AND(INDEX(REASON_NO_BED,3)&gt;INDEX(REASON_BEHAVIOR,3),INDEX(REASON_NO_BED,3)&gt;INDEX(REASON_SPECIAL_CARE,3),INDEX(REASON_NO_BED,3)&gt;INDEX(REASON_FINANCIAL,3),INDEX(REASON_NO_BED,3)&gt;INDEX(REASON_GUARDIANSHIP,3),INDEX(REASON_NO_BED,3)&gt;INDEX(REASON_PASARR,3),INDEX(REASON_NO_BED,3)&gt;INDEX(REASON_OTHER,3)),1,0)+IF(AND(INDEX(REASON_NO_BED,4)&gt;INDEX(REASON_BEHAVIOR,4),INDEX(REASON_NO_BED,4)&gt;INDEX(REASON_SPECIAL_CARE,4),INDEX(REASON_NO_BED,4)&gt;INDEX(REASON_FINANCIAL,4),INDEX(REASON_NO_BED,4)&gt;INDEX(REASON_GUARDIANSHIP,4),INDEX(REASON_NO_BED,4)&gt;INDEX(REASON_PASARR,4),INDEX(REASON_NO_BED,4)&gt;INDEX(REASON_OTHER,4)),1,0)+IF(AND(INDEX(REASON_NO_BED,5)&gt;INDEX(REASON_BEHAVIOR,5),INDEX(REASON_NO_BED,5)&gt;INDEX(REASON_SPECIAL_CARE,5),INDEX(REASON_NO_BED,5)&gt;INDEX(REASON_FINANCIAL,5),INDEX(REASON_NO_BED,5)&gt;INDEX(REASON_GUARDIANSHIP,5),INDEX(REASON_NO_BED,5)&gt;INDEX(REASON_PASARR,5),INDEX(REASON_NO_BED,5)&gt;INDEX(REASON_OTHER,5)),1,0)+IF(AND(INDEX(REASON_NO_BED,6)&gt;INDEX(REASON_BEHAVIOR,6),INDEX(REASON_NO_BED,6)&gt;INDEX(REASON_SPECIAL_CARE,6),INDEX(REASON_NO_BED,6)&gt;INDEX(REASON_FINANCIAL,6),INDEX(REASON_NO_BED,6)&gt;INDEX(REASON_GUARDIANSHIP,6),INDEX(REASON_NO_BED,6)&gt;INDEX(REASON_PASARR,6),INDEX(REASON_NO_BED,6)&gt;INDEX(REASON_OTHER,6)),1,0)+IF(AND(INDEX(REASON_NO_BED,7)&gt;INDEX(REASON_BEHAVIOR,7),INDEX(REASON_NO_BED,7)&gt;INDEX(REASON_SPECIAL_CARE,7),INDEX(REASON_NO_BED,7)&gt;INDEX(REASON_FINANCIAL,7),INDEX(REASON_NO_BED,7)&gt;INDEX(REASON_GUARDIANSHIP,7),INDEX(REASON_NO_BED,7)&gt;INDEX(REASON_PASARR,7),INDEX(REASON_NO_BED,7)&gt;INDEX(REASON_OTHER,7)),1,0)+IF(AND(INDEX(REASON_NO_BED,8)&gt;INDEX(REASON_BEHAVIOR,8),INDEX(REASON_NO_BED,8)&gt;INDEX(REASON_SPECIAL_CARE,8),INDEX(REASON_NO_BED,8)&gt;INDEX(REASON_FINANCIAL,8),INDEX(REASON_NO_BED,8)&gt;INDEX(REASON_GUARDIANSHIP,8),INDEX(REASON_NO_BED,8)&gt;INDEX(REASON_PASARR,8),INDEX(REASON_NO_BED,8)&gt;INDEX(REASON_OTHER,8)),1,0)</f>
+        <v>5.0</v>
+      </c>
+      <c r="E64" s="3">
+        <f>T3_YEARS</f>
+        <v>5</v>
+      </c>
+      <c r="F64">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="G64" t="str">
+        <f>IF(AND(ISNUMBER(D64),ISNUMBER(E64)),IF(ABS(D64-E64)&lt;=F64,"PASS","FAIL"),"FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="29">
+        <f>8</f>
+        <v>8</v>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>I8</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>MEETS_BENCH is TRUE exactly when GAP_PER_PT &lt;= 0, every year</t>
+        </is>
+      </c>
+      <c r="D65" t="b">
+        <f>AND(INDEX(MEETS_BENCH,1)=(INDEX(GAP_PER_PT,1)&lt;=0),INDEX(MEETS_BENCH,2)=(INDEX(GAP_PER_PT,2)&lt;=0),INDEX(MEETS_BENCH,3)=(INDEX(GAP_PER_PT,3)&lt;=0),INDEX(MEETS_BENCH,4)=(INDEX(GAP_PER_PT,4)&lt;=0),INDEX(MEETS_BENCH,5)=(INDEX(GAP_PER_PT,5)&lt;=0),INDEX(MEETS_BENCH,6)=(INDEX(GAP_PER_PT,6)&lt;=0),INDEX(MEETS_BENCH,7)=(INDEX(GAP_PER_PT,7)&lt;=0),INDEX(MEETS_BENCH,8)=(INDEX(GAP_PER_PT,8)&lt;=0))</f>
+        <v>1</v>
+      </c>
+      <c r="E65" t="b">
+        <f>TRUE</f>
+        <v>1</v>
+      </c>
+      <c r="F65" t="str">
+        <f>"exact"</f>
+        <v>exact</v>
+      </c>
+      <c r="G65" t="str">
+        <f>IF(D65=E65,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="29">
         <f>9</f>
         <v>9</v>
       </c>
-      <c r="B61" s="2" t="inlineStr">
+      <c r="B66" s="2" t="inlineStr">
         <is>
           <t>I9</t>
         </is>
       </c>
-      <c r="C61" s="2" t="inlineStr">
+      <c r="C66" s="2" t="inlineStr">
         <is>
           <t>Every WorkedExample row reads "match"</t>
         </is>
       </c>
-      <c r="D61" s="3">
+      <c r="D66" s="3">
         <f>COUNTIF(WorkedExample!E29:E57,"match")</f>
         <v>29</v>
       </c>
-      <c r="E61" s="3">
+      <c r="E66" s="3">
         <f>ROWS(WorkedExample!E29:E57)</f>
         <v>29</v>
-      </c>
-      <c r="F61">
-        <f>0</f>
-        <v>0</v>
-      </c>
-      <c r="G61" t="str">
-        <f>IF(AND(ISNUMBER(D61),ISNUMBER(E61)),IF(ABS(D61-E61)&lt;=F61,"PASS","FAIL"),"FAIL")</f>
-        <v>PASS</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="4" t="inlineStr">
-        <is>
-          <t>Error scans (count of error values in each sheet's used range; part of ALL CHECKS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="5" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B64" s="5" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="C64" s="5" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="D64" s="5" t="inlineStr">
-        <is>
-          <t>Computed</t>
-        </is>
-      </c>
-      <c r="E64" s="5" t="inlineStr">
-        <is>
-          <t>Expected</t>
-        </is>
-      </c>
-      <c r="F64" s="5" t="inlineStr">
-        <is>
-          <t>Tolerance</t>
-        </is>
-      </c>
-      <c r="G64" s="5" t="inlineStr">
-        <is>
-          <t>Result</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="29">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="B65" s="2" t="inlineStr">
-        <is>
-          <t>Error scan</t>
-        </is>
-      </c>
-      <c r="C65" s="2" t="inlineStr">
-        <is>
-          <t>No error values: Inputs (A1:S86)</t>
-        </is>
-      </c>
-      <c r="D65" s="3">
-        <f>SUMPRODUCT(--ISERROR(Inputs!A1:S86))</f>
-        <v>0.0</v>
-      </c>
-      <c r="E65" s="3">
-        <f>0</f>
-        <v>0</v>
-      </c>
-      <c r="F65">
-        <f>0</f>
-        <v>0</v>
-      </c>
-      <c r="G65" t="str">
-        <f>IF(AND(ISNUMBER(D65),ISNUMBER(E65)),IF(ABS(D65-E65)&lt;=F65,"PASS","FAIL"),"FAIL")</f>
-        <v>PASS</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="29">
-        <f>2</f>
-        <v>2</v>
-      </c>
-      <c r="B66" s="2" t="inlineStr">
-        <is>
-          <t>Error scan</t>
-        </is>
-      </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>No error values: Waitlist (A1:V19)</t>
-        </is>
-      </c>
-      <c r="D66" s="3">
-        <f>SUMPRODUCT(--ISERROR(Waitlist!A1:V19))</f>
-        <v>0.0</v>
-      </c>
-      <c r="E66" s="3">
-        <f>0</f>
-        <v>0</v>
       </c>
       <c r="F66">
         <f>0</f>
@@ -4856,106 +4914,54 @@
         <v>PASS</v>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="29">
-        <f>3</f>
-        <v>3</v>
-      </c>
-      <c r="B67" s="2" t="inlineStr">
-        <is>
-          <t>Error scan</t>
-        </is>
-      </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>No error values: Cost (A1:F22)</t>
-        </is>
-      </c>
-      <c r="D67" s="3">
-        <f>SUMPRODUCT(--ISERROR(Cost!A1:F22))</f>
-        <v>0.0</v>
-      </c>
-      <c r="E67" s="3">
-        <f>0</f>
-        <v>0</v>
-      </c>
-      <c r="F67">
-        <f>0</f>
-        <v>0</v>
-      </c>
-      <c r="G67" t="str">
-        <f>IF(AND(ISNUMBER(D67),ISNUMBER(E67)),IF(ABS(D67-E67)&lt;=F67,"PASS","FAIL"),"FAIL")</f>
-        <v>PASS</v>
-      </c>
-    </row>
     <row r="68">
-      <c r="A68" s="29">
-        <f>4</f>
-        <v>4</v>
-      </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>Error scan</t>
-        </is>
-      </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>No error values: Tests (A1:F41)</t>
-        </is>
-      </c>
-      <c r="D68" s="3">
-        <f>SUMPRODUCT(--ISERROR(Tests!A1:F41))</f>
-        <v>0.0</v>
-      </c>
-      <c r="E68" s="3">
-        <f>0</f>
-        <v>0</v>
-      </c>
-      <c r="F68">
-        <f>0</f>
-        <v>0</v>
-      </c>
-      <c r="G68" t="str">
-        <f>IF(AND(ISNUMBER(D68),ISNUMBER(E68)),IF(ABS(D68-E68)&lt;=F68,"PASS","FAIL"),"FAIL")</f>
-        <v>PASS</v>
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>Error scans (count of error values in each sheet's used range; part of ALL CHECKS)</t>
+        </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="29">
-        <f>5</f>
-        <v>5</v>
-      </c>
-      <c r="B69" s="2" t="inlineStr">
-        <is>
-          <t>Error scan</t>
-        </is>
-      </c>
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>No error values: County (A1:F12)</t>
-        </is>
-      </c>
-      <c r="D69" s="3">
-        <f>SUMPRODUCT(--ISERROR(County!A1:F12))</f>
-        <v>0.0</v>
-      </c>
-      <c r="E69" s="3">
-        <f>0</f>
-        <v>0</v>
-      </c>
-      <c r="F69">
-        <f>0</f>
-        <v>0</v>
-      </c>
-      <c r="G69" t="str">
-        <f>IF(AND(ISNUMBER(D69),ISNUMBER(E69)),IF(ABS(D69-E69)&lt;=F69,"PASS","FAIL"),"FAIL")</f>
-        <v>PASS</v>
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>Computed</t>
+        </is>
+      </c>
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="F69" s="5" t="inlineStr">
+        <is>
+          <t>Tolerance</t>
+        </is>
+      </c>
+      <c r="G69" s="5" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="29">
-        <f>6</f>
-        <v>6</v>
+        <f>1</f>
+        <v>1</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
@@ -4964,11 +4970,11 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>No error values: Capacity (A1:E22)</t>
+          <t>No error values: Inputs (A1:S86)</t>
         </is>
       </c>
       <c r="D70" s="3">
-        <f>SUMPRODUCT(--ISERROR(Capacity!A1:E22))</f>
+        <f>SUMPRODUCT(--ISERROR(Inputs!A1:S86))</f>
         <v>0.0</v>
       </c>
       <c r="E70" s="3">
@@ -4986,8 +4992,8 @@
     </row>
     <row r="71">
       <c r="A71" s="29">
-        <f>7</f>
-        <v>7</v>
+        <f>2</f>
+        <v>2</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
@@ -4996,11 +5002,11 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>No error values: Conditions (A1:F17)</t>
+          <t>No error values: Waitlist (A1:V19)</t>
         </is>
       </c>
       <c r="D71" s="3">
-        <f>SUMPRODUCT(--ISERROR(Conditions!A1:F17))</f>
+        <f>SUMPRODUCT(--ISERROR(Waitlist!A1:V19))</f>
         <v>0.0</v>
       </c>
       <c r="E71" s="3">
@@ -5018,8 +5024,8 @@
     </row>
     <row r="72">
       <c r="A72" s="29">
-        <f>8</f>
-        <v>8</v>
+        <f>3</f>
+        <v>3</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
@@ -5028,11 +5034,11 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>No error values: FigureData (A1:J88)</t>
+          <t>No error values: Cost (A1:F22)</t>
         </is>
       </c>
       <c r="D72" s="3">
-        <f>SUMPRODUCT(--ISERROR(FigureData!A1:J88))</f>
+        <f>SUMPRODUCT(--ISERROR(Cost!A1:F22))</f>
         <v>0.0</v>
       </c>
       <c r="E72" s="3">
@@ -5050,8 +5056,8 @@
     </row>
     <row r="73">
       <c r="A73" s="29">
-        <f>9</f>
-        <v>9</v>
+        <f>4</f>
+        <v>4</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
@@ -5060,11 +5066,11 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>No error values: WorkedExample (A1:G62)</t>
+          <t>No error values: Tests (A1:F41)</t>
         </is>
       </c>
       <c r="D73" s="3">
-        <f>SUMPRODUCT(--ISERROR(WorkedExample!A1:G62))</f>
+        <f>SUMPRODUCT(--ISERROR(Tests!A1:F41))</f>
         <v>0.0</v>
       </c>
       <c r="E73" s="3">
@@ -5082,8 +5088,8 @@
     </row>
     <row r="74">
       <c r="A74" s="29">
-        <f>10</f>
-        <v>10</v>
+        <f>5</f>
+        <v>5</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
@@ -5092,11 +5098,11 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>No error values: Checks (rows 1 to 73, above this row)</t>
+          <t>No error values: County (A1:F12)</t>
         </is>
       </c>
       <c r="D74" s="3">
-        <f>SUMPRODUCT(--ISERROR(A1:G73))</f>
+        <f>SUMPRODUCT(--ISERROR(County!A1:F12))</f>
         <v>0.0</v>
       </c>
       <c r="E74" s="3">
@@ -5112,34 +5118,194 @@
         <v>PASS</v>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" s="29">
+        <f>6</f>
+        <v>6</v>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Error scan</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>No error values: Capacity (A1:E22)</t>
+        </is>
+      </c>
+      <c r="D75" s="3">
+        <f>SUMPRODUCT(--ISERROR(Capacity!A1:E22))</f>
+        <v>0.0</v>
+      </c>
+      <c r="E75" s="3">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="F75">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="G75" t="str">
+        <f>IF(AND(ISNUMBER(D75),ISNUMBER(E75)),IF(ABS(D75-E75)&lt;=F75,"PASS","FAIL"),"FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
     <row r="76">
+      <c r="A76" s="29">
+        <f>7</f>
+        <v>7</v>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Error scan</t>
+        </is>
+      </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
+          <t>No error values: Conditions (A1:F38)</t>
+        </is>
+      </c>
+      <c r="D76" s="3">
+        <f>SUMPRODUCT(--ISERROR(Conditions!A1:F38))</f>
+        <v>0.0</v>
+      </c>
+      <c r="E76" s="3">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="F76">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="G76" t="str">
+        <f>IF(AND(ISNUMBER(D76),ISNUMBER(E76)),IF(ABS(D76-E76)&lt;=F76,"PASS","FAIL"),"FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="29">
+        <f>8</f>
+        <v>8</v>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Error scan</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>No error values: FigureData (A1:J88)</t>
+        </is>
+      </c>
+      <c r="D77" s="3">
+        <f>SUMPRODUCT(--ISERROR(FigureData!A1:J88))</f>
+        <v>0.0</v>
+      </c>
+      <c r="E77" s="3">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="F77">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="G77" t="str">
+        <f>IF(AND(ISNUMBER(D77),ISNUMBER(E77)),IF(ABS(D77-E77)&lt;=F77,"PASS","FAIL"),"FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="29">
+        <f>9</f>
+        <v>9</v>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Error scan</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>No error values: WorkedExample (A1:G62)</t>
+        </is>
+      </c>
+      <c r="D78" s="3">
+        <f>SUMPRODUCT(--ISERROR(WorkedExample!A1:G62))</f>
+        <v>0.0</v>
+      </c>
+      <c r="E78" s="3">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="F78">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="G78" t="str">
+        <f>IF(AND(ISNUMBER(D78),ISNUMBER(E78)),IF(ABS(D78-E78)&lt;=F78,"PASS","FAIL"),"FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="29">
+        <f>10</f>
+        <v>10</v>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Error scan</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>No error values: Checks (rows 1 to 78, above this row)</t>
+        </is>
+      </c>
+      <c r="D79" s="3">
+        <f>SUMPRODUCT(--ISERROR(A1:G78))</f>
+        <v>0.0</v>
+      </c>
+      <c r="E79" s="3">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="F79">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="G79" t="str">
+        <f>IF(AND(ISNUMBER(D79),ISNUMBER(E79)),IF(ABS(D79-E79)&lt;=F79,"PASS","FAIL"),"FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="C81" s="2" t="inlineStr">
+        <is>
           <t>ALL CHECKS (invariants and error scans)</t>
         </is>
       </c>
-      <c r="D76" s="4" t="str">
-        <f>IF(AND(COUNTIF(G53:G61,"FAIL")+COUNTIF(G65:G74,"FAIL")=0,COUNTIF(G53:G61,"PASS")+COUNTIF(G65:G74,"PASS")=19),"ALL PASS","REVIEW")</f>
+      <c r="D81" s="4" t="str">
+        <f>IF(AND(COUNTIF(G58:G66,"FAIL")+COUNTIF(G70:G79,"FAIL")=0,COUNTIF(G58:G66,"PASS")+COUNTIF(G70:G79,"PASS")=19),"ALL PASS","REVIEW")</f>
         <v>ALL PASS</v>
       </c>
     </row>
-    <row r="77">
-      <c r="C77" s="2" t="inlineStr">
+    <row r="82">
+      <c r="C82" s="2" t="inlineStr">
         <is>
           <t>Anchors matching</t>
         </is>
       </c>
-      <c r="D77" s="3">
-        <f>COUNTIF(G5:G49,"PASS")</f>
-        <v>45</v>
-      </c>
-      <c r="E77" t="str">
-        <f>"of "&amp;ROWS(G5:G49)</f>
-        <v>of 45</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="16" t="inlineStr">
+      <c r="D82" s="3">
+        <f>COUNTIF(G5:G54,"PASS")</f>
+        <v>50</v>
+      </c>
+      <c r="E82" t="str">
+        <f>"of "&amp;ROWS(G5:G54)</f>
+        <v>of 50</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="16" t="inlineStr">
         <is>
           <t>Anchor tolerance = half a unit of the spec's shown precision; invariant tolerance 1e-6. Checked outside the workbook by script (spec Audit findings): every calculated cell is a formula; every spec name exists as an absolute defined name and no others; every input cell is yellow and no calculated cell is.</t>
         </is>
@@ -7377,13 +7543,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="88" customWidth="1" style="7" min="1" max="1"/>
-    <col width="14" customWidth="1" style="7" min="2" max="2"/>
+    <col width="16" customWidth="1" style="7" min="2" max="2"/>
     <col width="20" customWidth="1" style="7" min="3" max="3"/>
-    <col width="16" customWidth="1" style="7" min="4" max="4"/>
+    <col width="22" customWidth="1" style="7" min="4" max="4"/>
     <col width="22" customWidth="1" style="7" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -7565,6 +7731,249 @@
       <c r="A15" s="16" t="inlineStr">
         <is>
           <t>Not a forecast; the model does not rank or cost the options (spec Conventions, Condition (a)).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Paper figures: the rate against Medicaid-heavy cost, the two rate rises, and the behavior and guardianship share</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="45" customHeight="1" s="7">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Fiscal year</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>July rate median</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Medicaid-heavy cost</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Gap, 1 - rate / cost (RATE_COST_GAP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>FY2016</t>
+        </is>
+      </c>
+      <c r="B19" s="35">
+        <f>IF(IF(ISNUMBER(MATCH(DATE(2016,7,1),RATE_DATE,0)),ISNUMBER(INDEX(NF_RATE_MEDIAN,MATCH(DATE(2016,7,1),RATE_DATE,0))),FALSE),INDEX(NF_RATE_MEDIAN,MATCH(DATE(2016,7,1),RATE_DATE,0)),"")</f>
+        <v>252.4</v>
+      </c>
+      <c r="C19" s="35">
+        <f>INDEX(NF_COST_MCD_HEAVY,MATCH(2016,COST_FY,0))</f>
+        <v>344.38</v>
+      </c>
+      <c r="D19" s="26">
+        <f>IF(ISNUMBER(B19),1-B19/C19,"")</f>
+        <v>0.26708868110807826</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>FY2017</t>
+        </is>
+      </c>
+      <c r="B20" s="35">
+        <f>IF(IF(ISNUMBER(MATCH(DATE(2017,7,1),RATE_DATE,0)),ISNUMBER(INDEX(NF_RATE_MEDIAN,MATCH(DATE(2017,7,1),RATE_DATE,0))),FALSE),INDEX(NF_RATE_MEDIAN,MATCH(DATE(2017,7,1),RATE_DATE,0)),"")</f>
+        <v>261.45</v>
+      </c>
+      <c r="C20" s="35">
+        <f>INDEX(NF_COST_MCD_HEAVY,MATCH(2017,COST_FY,0))</f>
+        <v>356.1</v>
+      </c>
+      <c r="D20" s="26">
+        <f>IF(ISNUMBER(B20),1-B20/C20,"")</f>
+        <v>0.26579612468407754</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>FY2018</t>
+        </is>
+      </c>
+      <c r="B21" s="35">
+        <f>IF(IF(ISNUMBER(MATCH(DATE(2018,7,1),RATE_DATE,0)),ISNUMBER(INDEX(NF_RATE_MEDIAN,MATCH(DATE(2018,7,1),RATE_DATE,0))),FALSE),INDEX(NF_RATE_MEDIAN,MATCH(DATE(2018,7,1),RATE_DATE,0)),"")</f>
+        <v>270.66</v>
+      </c>
+      <c r="C21" s="35">
+        <f>INDEX(NF_COST_MCD_HEAVY,MATCH(2018,COST_FY,0))</f>
+        <v>365.93</v>
+      </c>
+      <c r="D21" s="26">
+        <f>IF(ISNUMBER(B21),1-B21/C21,"")</f>
+        <v>0.2603503402290055</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>FY2019</t>
+        </is>
+      </c>
+      <c r="B22" s="35" t="str">
+        <f>IF(IF(ISNUMBER(MATCH(DATE(2019,7,1),RATE_DATE,0)),ISNUMBER(INDEX(NF_RATE_MEDIAN,MATCH(DATE(2019,7,1),RATE_DATE,0))),FALSE),INDEX(NF_RATE_MEDIAN,MATCH(DATE(2019,7,1),RATE_DATE,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C22" s="35">
+        <f>INDEX(NF_COST_MCD_HEAVY,MATCH(2019,COST_FY,0))</f>
+        <v>373.25</v>
+      </c>
+      <c r="D22" s="26" t="str">
+        <f>IF(ISNUMBER(B22),1-B22/C22,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>FY2020</t>
+        </is>
+      </c>
+      <c r="B23" s="35">
+        <f>IF(IF(ISNUMBER(MATCH(DATE(2020,7,1),RATE_DATE,0)),ISNUMBER(INDEX(NF_RATE_MEDIAN,MATCH(DATE(2020,7,1),RATE_DATE,0))),FALSE),INDEX(NF_RATE_MEDIAN,MATCH(DATE(2020,7,1),RATE_DATE,0)),"")</f>
+        <v>282.98</v>
+      </c>
+      <c r="C23" s="35">
+        <f>INDEX(NF_COST_MCD_HEAVY,MATCH(2020,COST_FY,0))</f>
+        <v>398.33</v>
+      </c>
+      <c r="D23" s="26">
+        <f>IF(ISNUMBER(B23),1-B23/C23,"")</f>
+        <v>0.289584013255341</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
+      <c r="B24" s="35">
+        <f>IF(IF(ISNUMBER(MATCH(DATE(2021,7,1),RATE_DATE,0)),ISNUMBER(INDEX(NF_RATE_MEDIAN,MATCH(DATE(2021,7,1),RATE_DATE,0))),FALSE),INDEX(NF_RATE_MEDIAN,MATCH(DATE(2021,7,1),RATE_DATE,0)),"")</f>
+        <v>334.75</v>
+      </c>
+      <c r="C24" s="35">
+        <f>INDEX(NF_COST_MCD_HEAVY,MATCH(2021,COST_FY,0))</f>
+        <v>423.44</v>
+      </c>
+      <c r="D24" s="26">
+        <f>IF(ISNUMBER(B24),1-B24/C24,"")</f>
+        <v>0.20945116191195923</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="B25" s="35" t="str">
+        <f>IF(IF(ISNUMBER(MATCH(DATE(2022,7,1),RATE_DATE,0)),ISNUMBER(INDEX(NF_RATE_MEDIAN,MATCH(DATE(2022,7,1),RATE_DATE,0))),FALSE),INDEX(NF_RATE_MEDIAN,MATCH(DATE(2022,7,1),RATE_DATE,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C25" s="35">
+        <f>INDEX(NF_COST_MCD_HEAVY,MATCH(2022,COST_FY,0))</f>
+        <v>435.63</v>
+      </c>
+      <c r="D25" s="26" t="str">
+        <f>IF(ISNUMBER(B25),1-B25/C25,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="B26" s="35">
+        <f>IF(IF(ISNUMBER(MATCH(DATE(2023,7,1),RATE_DATE,0)),ISNUMBER(INDEX(NF_RATE_MEDIAN,MATCH(DATE(2023,7,1),RATE_DATE,0))),FALSE),INDEX(NF_RATE_MEDIAN,MATCH(DATE(2023,7,1),RATE_DATE,0)),"")</f>
+        <v>371.99</v>
+      </c>
+      <c r="C26" s="35">
+        <f>INDEX(NF_COST_MCD_HEAVY,MATCH(2023,COST_FY,0))</f>
+        <v>461.79</v>
+      </c>
+      <c r="D26" s="26">
+        <f>IF(ISNUMBER(B26),1-B26/C26,"")</f>
+        <v>0.19446068559301843</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Smallest gap, FY2016 to FY2023 (RATE_COST_GAP_MIN)</t>
+        </is>
+      </c>
+      <c r="B28" s="26">
+        <f>MIN(D19:D26)</f>
+        <v>0.19446068559301843</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Largest gap, FY2016 to FY2023 (RATE_COST_GAP_MAX)</t>
+        </is>
+      </c>
+      <c r="B29" s="26">
+        <f>MAX(D19:D26)</f>
+        <v>0.289584013255341</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Rate rise, July 2020 to July 2021 (RATE_RISE_2021)</t>
+        </is>
+      </c>
+      <c r="B31" s="20">
+        <f>INDEX(NF_RATE_MEDIAN,MATCH(DATE(2021,7,1),RATE_DATE,0))/INDEX(NF_RATE_MEDIAN,MATCH(DATE(2020,7,1),RATE_DATE,0))-1</f>
+        <v>0.1829457912219945</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Rate rise, July 2023 to January 2024 (RATE_RISE_2024)</t>
+        </is>
+      </c>
+      <c r="B32" s="20">
+        <f>INDEX(NF_RATE_MEDIAN,MATCH(DATE(2024,1,1),RATE_DATE,0))/INDEX(NF_RATE_MEDIAN,MATCH(DATE(2023,7,1),RATE_DATE,0))-1</f>
+        <v>0.29527675475147164</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Behavior and guardianship share, Dec 31, 2024 (BEH_GUARD_SHARE_2024)</t>
+        </is>
+      </c>
+      <c r="B34" s="20">
+        <f>INDEX(SHARE_BEHAVIOR,MATCH(2024,YEAR,0))+INDEX(SHARE_GUARDIANSHIP,MATCH(2024,YEAR,0))</f>
+        <v>0.3468208092485549</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="16" t="inlineStr">
+        <is>
+          <t>The gap pairs each fiscal year's cost with that July's rate memo; years with no July median in the rate series (2019, 2022) are blank. The rate median covers all homes; the cost median covers Medicaid-heavy homes.</t>
         </is>
       </c>
     </row>

</xml_diff>